<commit_message>
Executive deck (28 slides, pptx/pdf, validated); LinkedIn series complete (24 posts + 3 reactive templates); content calendar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYt6k15P64MhHqeyveeQ6D
</commit_message>
<xml_diff>
--- a/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
+++ b/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1957,9 +1957,471 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D22" s="5">
+        <f>IF($E$1="","",$E$1+63)</f>
+        <v/>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>The worked example, end to end</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Post 20 (Start small, Week 10 Thursday). **Bridge:** Tuesday shows the full worked example and its "never" list; Thursday shows the minimum platform needed to run it, and what to leave out.</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>What the attribution-commentary agent must never do matters more than what it can do.</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>For nine weeks one example has run underneath this series: an agent that drafts the monthly performance-attribution commentary for a multi-asset fund, with a portfolio manager approving every draft. It is generic and illustrative. Here it is in one place.</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>265</v>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>#AgenticAI #AIGovernance</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Two-column "may / must never" table for the worked example. Each "never" row has its enforcing component in a coloured chip (read-only tool, numeric comparator, approval interrupt, allow-list, tokenisation, entitlement filter, version pin). Beneath it, the eight-tile evidence pack keyed to one trace ID. Source: synthesis VI.3 and VI.4. Label: "generic, illustrative".</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>- No product or regulatory facts in the body. Check that the first comment's per-cloud examples match the final document.</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="P22" s="4" t="inlineStr"/>
+      <c r="Q22" s="4" t="inlineStr"/>
+      <c r="R22" s="4" t="inlineStr">
+        <is>
+          <t>Master_Architecture: LinkedIn series, Post 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D23" s="5">
+        <f>IF($E$1="","",$E$1+65)</f>
+        <v/>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Start small</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Post 19 (Worked example, Week 10 Tuesday). **Bridge:** Tuesday's agent needs a platform; Thursday argues that the minimum platform, plus a published "not yet" list, is the right first release.</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>The most valuable part of a reference architecture is the "do not build yet" list.</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>The most valuable page in a reference architecture is often the "do not build yet" list.</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>264</v>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>#EnterpriseArchitecture #AgenticAI</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Two panels. Left, "Build now": the Stack D minimum as a compact stack (gateway ×2, identity, manifest, checks, eval suite, one store, one workflow, two models). Right, "Do NOT build yet": the not-yet items as greyed-out tiles, each with a one-word trigger for revisiting it ("evidence", "load test", "use case"). Source: synthesis Part VII, Stack D.</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>- The not-yet list against the final Part VII and the Part XI tiers (anything promoted from Experimental)</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="P23" s="4" t="inlineStr"/>
+      <c r="Q23" s="4" t="inlineStr"/>
+      <c r="R23" s="4" t="inlineStr">
+        <is>
+          <t>Master_Architecture: LinkedIn series, Post 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D24" s="5">
+        <f>IF($E$1="","",$E$1+70)</f>
+        <v/>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Build vs buy</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Post 22 (Where not to abstract, Week 11 Thursday). **Bridge:** Tuesday says to own a thin interface in front of what you buy; Thursday warns against owning too many interfaces.</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Build where you differentiate, buy where you would only be maintaining.</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Build where you differentiate. Buy where you would only be maintaining.</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>257</v>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>#EnterpriseArchitecture #BuildVsBuy</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Three-column board, "Build · Hybrid · Buy", with the 17 layers and controls placed as cards (for example, Build: tool servers, configuration of record, evidence store; Hybrid: gateway, guardrails, privacy, evaluation, retrieval optimisation; Buy: security tooling, foundation models, serving access). A separate red card reads "Do not build yet: fine-tuning". Source: synthesis Part VIII table.</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>- No dated facts in the body. Check the Article 25 wording if challenged ("can, in some cases").</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr"/>
+      <c r="Q24" s="4" t="inlineStr"/>
+      <c r="R24" s="4" t="inlineStr">
+        <is>
+          <t>Master_Architecture: LinkedIn series, Post 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D25" s="5">
+        <f>IF($E$1="","",$E$1+72)</f>
+        <v/>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Where not to abstract</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Post 21 (Build vs buy, Week 11 Tuesday). **Bridge:** Tuesday's thin firm-owned interfaces are the right default; Thursday names where adding one is the mistake.</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Frameworks on top of frameworks.</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Abstraction is how an architecture stays reversible. Too much of it is how an architecture stops moving.</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>253</v>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>#SoftwareArchitecture #AgenticAI</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Two lists side by side. "Abstract (thin, firm-owned)": routing contract, telemetry collector, datasets, credentials, policy, retrieval interface, embed/rerank, privacy API, memory API, config fetch. "Do not over-abstract": agent frameworks, single-workflow plug-ins, plain database access, store-bundled features, vendor model extras. A small strip beneath shows "multi-vendor necessary" versus "multi-vendor only adds complexity". Source: synthesis IX.1–IX.3.</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>- No dated facts in the body.</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="P25" s="4" t="inlineStr"/>
+      <c r="Q25" s="4" t="inlineStr"/>
+      <c r="R25" s="4" t="inlineStr">
+        <is>
+          <t>Master_Architecture: LinkedIn series, Post 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D26" s="5">
+        <f>IF($E$1="","",$E$1+77)</f>
+        <v/>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Which lock-in is acceptable</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Post 24 (Close, Week 12 Thursday). **Bridge:** Tuesday classifies which dependencies are worth accepting; Thursday applies that to the final stack: what I would select, and what I would deliberately leave out.</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Some lock-in is a good trade, and the skill is knowing which.</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>Some lock-in is a good trade. The skill is knowing which.</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>257</v>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>#VendorRisk #EnterpriseArchitecture</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Heat-map table: the 17 layers and controls as rows; columns "acceptable", "manageable", "unacceptable"; each cell a short phrase from the synthesis table (vendor names removed). A highlighted band across the "unacceptable" column reads "the firm's own records: evidence, configuration, datasets, credentials". Source: synthesis IX.4.</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>- Lock-in categories against the final Part IX.4 table - Any new ownership change in a "manageable" category</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="P26" s="4" t="inlineStr"/>
+      <c r="Q26" s="4" t="inlineStr"/>
+      <c r="R26" s="4" t="inlineStr">
+        <is>
+          <t>Master_Architecture: LinkedIn series, Post 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D27" s="5">
+        <f>IF($E$1="","",$E$1+79)</f>
+        <v/>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Close: what I'd select, and what I'd deliberately not select</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Post 23 (Which lock-in is acceptable, Week 12 Tuesday). **Bridge:** Tuesday's lock-in classification is the filter; Thursday shows what passes through it, what does not, and what leading the change actually requires.</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>The full stack on one page, plus a lesson about leading the transformation.</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Twelve weeks ago this series started from a popular diagram of the AI stack. On this review, 39 of its 80 product tiles were out of date. The diagram was a catalogue. The enterprise problem is a control system.</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>269</v>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>#EnterpriseArchitecture #AIGovernance</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>The one-page architecture from synthesis I.2, with vendor names removed: control plane (C1–C8 with the L9 evidence plane) across the top; agent, knowledge and model planes beneath. To the right, a short "Deliberately not selected" column with the categories from XI.5 and XI.7. Optional carousel: slide 1 the original diagram with 39 tiles flagged; slide 2 the one-page architecture; slide 3 the twelve decisions; slide 4 "not selected".</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>- The final Part XI lists (avoid and monitor), especially any item that has changed tier since October 2026 - Ownership and status changes across the products in the first comment</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="P27" s="4" t="inlineStr"/>
+      <c r="Q27" s="4" t="inlineStr"/>
+      <c r="R27" s="4" t="inlineStr">
+        <is>
+          <t>Master_Architecture: LinkedIn series, Post 24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="N4:N21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N4:N27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Draft,Anecdote added,Scheduled,Published,Skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Print/Kindle edition tooling, rebuild script, updated run guides, LinkedIn visuals in the series document
- tools/build_print_edition.py + tools/print/print_pdf.py + tools/print/book.json: KDP-ready interior, cover wrap, EPUB, build summary, publishing kit
- tools/rebuild_all.sh: rebuild every deliverable in order; deck theme writer made portable
- RERUN_ON_DESKTOP.md and REFRESH_QUARTERLY.md updated for the new toolchain; CONTEXT/CLAUDE house conventions extended (one home per section, the book)
- Synthesis: I.4 references corrected to I.3, XII.1 points to what_changed.xlsx; MEMORY run log 31-35

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYt6k15P64MhHqeyveeQ6D
</commit_message>
<xml_diff>
--- a/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
+++ b/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -567,24 +567,24 @@
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>Full post (master document)</t>
+          <t>Full post and visual</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D4" s="5">
-        <f>IF($E$1="","",$E$1+0)</f>
+        <f>IF($E$1="","",$E$1+-5)</f>
         <v/>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -594,40 +594,40 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>L9 Evaluation and observability</t>
+          <t>Series introduction: the enterprise GenAI stack, layer by layer</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Post 2 (C8, Week 1 Thursday). **Bridge:** Tuesday argues that evaluation must exist from day one; Thursday shows that the same eval suite, run independently and kept, is the validation evidence a model-risk function needs.</t>
+          <t>Post 1 (L1, Week 1 Tuesday). **Bridge:** The series starts where every architecture starts: the models, and how not to bet the firm on one of them.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>The layer that ages slowest is the one most teams build last, and evals added after go-live measure the damage, not the quality.</t>
+          <t>The logos move faster than any diagram; the controls around them are what last.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Most diagrams of the AI stack put evaluation in the last box. It is the layer that ages slowest — and the one most teams build last.</t>
+          <t>Over the next twelve weeks I am going to take the enterprise GenAI stack apart, one layer at a time.</t>
         </is>
       </c>
       <c r="J4" s="4" t="n">
-        <v>261</v>
+        <v>232</v>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>#AIEvaluation #LLMOps</t>
+          <t>#GenerativeAI #EnterpriseArchitecture</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Two-panel diagram. Left: the original nine-layer stack with "Evals and observability" as the last box. Right: the same stack with evaluation and observability redrawn as a vertical plane running alongside every layer, labelled "firm-owned telemetry and evidence spine", with products drawn as replaceable plug-ins. A small callout shows the one metric: "Numeric faithfulness: 100%, any miss blocks." Source: L9 §9.13 and the H8 provisional view.</t>
+          <t>Series map: the nine layers (L1 → L9) as a stack on the left, each paired by a connector with its Thursday control or theme on the right, labelled with week numbers 1–9. Weeks 10–12 (worked example, start small, build vs buy, where not to abstract, lock-in, close) as a strip beneath. A banner across the top: "the control plane around the products is the architecture". Footer: "24 posts · 12 weeks · one worked example". Source: the calendar above and synthesis Part I.</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>- Arize/Dynatrace completion and the Langfuse/ClickHouse status - Whether OpenAI's Promptfoo acquisition has closed - OpenTelemetry GenAI conventions still at "Development" - The "five of the eleven" count, against the final L9 table</t>
+          <t>- The counts (140 products, 1,255 sources, 39 of 80 tiles) against the final published edition - The start date of Post 1 (the first Tuesday after sign-off)</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
@@ -644,24 +644,24 @@
       <c r="Q4" s="4" t="inlineStr"/>
       <c r="R4" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 1</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 0 · visual 08_Graphic/linkedin/P00.png</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D5" s="5">
-        <f>IF($E$1="","",$E$1+2)</f>
+        <f>IF($E$1="","",$E$1+0)</f>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -671,40 +671,40 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>C8 Model risk, governance and audit</t>
+          <t>L1 Foundation models</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Post 1 (L9, Week 1 Tuesday). **Bridge:** Tuesday's eval suite becomes Thursday's validation evidence, but only if someone independent challenges it, it is versioned, and it is retained.</t>
+          <t>Post 2 (C6, Week 1 Thursday). **Bridge:** A portfolio of models needs a way to choose between them on cost without fooling yourself; Thursday supplies the metric.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Your eval suite *is* your validation evidence. What model-risk discipline means when the "model" is an agent and the main US guidance has stepped aside.</t>
+          <t>Treat models as a portfolio, not a bet.</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>In April, the US supervisory guidance that had shaped model risk management since 2011 was replaced. Its successor, SR 26-2, places generative and agentic AI expressly outside its scope.</t>
+          <t>Treat foundation models as a portfolio, not a bet.</t>
         </is>
       </c>
       <c r="J5" s="4" t="n">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>#ModelRisk #AIGovernance</t>
+          <t>#FoundationModels #VendorRisk</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>One-page "evidence pack" graphic for the worked example: eight tiles (prompt version, model version, data snapshot, tool calls, eval results, approver identity, timestamps, final output), all keyed to one trace ID and feeding an immutable archive. A side panel shows "governed unit = use case" with the model as a vendor component. Source: C8 §C8.12.</t>
+          <t>Portfolio grid: four roles (primary mid tier, fallback mid tier from a different vendor, small classifier, self-hosted open weight) as rows, with columns "pinned version", "region", "qualified on eval suite (date)", "retirement runway". All rows feed one gateway. A "frontier tier: off by default" tile sits above. Source: L1 §1.9 and §1.12 (shown without vendor names).</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>- SR 26-2 status, and whether the agencies' AI/GenAI request for information has been published (update the post if it has) - SS1/23 scope statements - Collibra–trail ML completion</t>
+          <t>- The Gemini Flash retirement date and the Claude Fable 5 suspension dates (both cited in the first comment) - Current model families and versions, which change monthly - CP4 tier decisions as published in the final document</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
@@ -721,24 +721,24 @@
       <c r="Q5" s="4" t="inlineStr"/>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 2</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 1 · visual 08_Graphic/linkedin/P01.png</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D6" s="5">
-        <f>IF($E$1="","",$E$1+7)</f>
+        <f>IF($E$1="","",$E$1+2)</f>
         <v/>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -748,40 +748,40 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>L8 Data extraction and ingestion</t>
+          <t>C6 AI FinOps</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Post 4 (C3, Week 2 Thursday). **Bridge:** Tuesday shows that quality is decided at ingestion; Thursday shows that residency and privacy are decided there too.</t>
+          <t>Post 1 (L1, Week 1 Tuesday). **Bridge:** A model portfolio is only as good as the cost metric used to choose within it, and cost per token is the wrong one.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Some of the most convincing "hallucinations" in enterprise retrieval start in a PDF table parser, not in the model.</t>
+          <t>Cost per task, not cost per token, is the metric executives understand.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Some of the most convincing "hallucinations" in enterprise retrieval systems are not the model's fault. They start in a table parser.</t>
+          <t>Cost per token is the number on the price list. Cost per task is the number executives understand, and the one that tells you whether a change saved anything.</t>
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>236</v>
+        <v>262</v>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>#RAG #DataQuality</t>
+          <t>#FinOps #UnitEconomics</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Pipeline diagram: source register → acquisition → classification/DLP → parser (drawn as a swappable cartridge) → "metadata envelope" stamped on each chunk (source, version, ACL, classification, parser manifest, lineage ID) → index gate ("no envelope, no index"). A red side-path shows "parsed numbers = context only"; a green path shows "authoritative figures via read-only tool". Source: L8 §8.9 and the six-component control plane in §8.13.</t>
+          <t>Side-by-side bars for one approved commentary (illustrative): "token cost" (small) versus "reviewer time" (large), with a third bar "regenerations" that multiplies the token cost. Beneath, the data flow: gateway meter (tags: use case, fund, run ID) → join to trace → monthly reconciliation to invoice → firm-owned cost dataset. Label clearly as illustrative. Source: C6 §C6.9 and §C6.12.</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>- "Ten products assessed; only one carries ACL metadata; none emits lineage" (check for new lineage features) - Mistral OCR and Docling version status if mentioned in replies</t>
+          <t>- List prices used in the illustrative arithmetic (they change often; "well under a dollar" should still hold) - FOCUS 1.5 ratification status</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
@@ -798,24 +798,24 @@
       <c r="Q6" s="4" t="inlineStr"/>
       <c r="R6" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 3</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 2 · visual 08_Graphic/linkedin/P02.png</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D7" s="5">
-        <f>IF($E$1="","",$E$1+9)</f>
+        <f>IF($E$1="","",$E$1+7)</f>
         <v/>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -825,40 +825,40 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>C3 DLP and PII protection</t>
+          <t>L2 Inference, serving and model access</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Post 3 (L8, Week 2 Tuesday). **Bridge:** If quality is decided at ingestion, so are residency and privacy; a filter at the prompt arrives too late.</t>
+          <t>Post 4 (C1, Week 2 Thursday). **Bridge:** Tuesday makes managed access the default; Thursday shows the gateway is what keeps that choice reversible.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Data residency and PII decisions are made at ingestion, not at the prompt.</t>
+          <t>Self-hosting is a capacity and operating-model decision, not just a cost decision.</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>One analyst question can place the same client identifier in seven places: a prompt, a retrieved chunk, a tool result, a provider's processing region, a trace store, an evaluation dataset and a memory record.</t>
+          <t>Self-hosting a model is a capacity and operating-model decision. It is only partly a cost decision.</t>
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>#DataProtection #PrivacyEngineering</t>
+          <t>#LLMInference #MLOps</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>"Seven copies" diagram: one client identifier at the centre with arrows to seven stores (prompt, chunk, tool result, provider region, trace store, eval set, memory). Overlay six numbered enforcement points (E1 ingestion to E6 trace export) all calling one "privacy service" box. Inset: a draft showing CLIENT_A / MANDATE_1 placeholders instead of names. Source: C3 §C3.2, §C3.9 step 0, §C3.12.</t>
+          <t>L2 split into three stacked sub-layers (serving engines; optimisation, marked "only if you run GPU fleets"; model access), with the gateway lifted out into the control plane. Beside it, a month-end demand curve against a reserved-capacity line, showing headroom and an "overflow stays in region" arrow. Source: L2 §2.3, §2.9 step 3, §2.13 H1 view.</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>- Status of the DPF appeal C-703/25 P - Presidio governance and licence - Purview DSPM licensing statement</t>
+          <t>- Overflow and residency behaviour statements for each hyperscaler - OpenRouter–Stripe closing; SGLang advisory status</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -875,24 +875,24 @@
       <c r="Q7" s="4" t="inlineStr"/>
       <c r="R7" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 4</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 3 · visual 08_Graphic/linkedin/P03.png</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D8" s="5">
-        <f>IF($E$1="","",$E$1+14)</f>
+        <f>IF($E$1="","",$E$1+9)</f>
         <v/>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -902,40 +902,40 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>L7 Embeddings and reranking</t>
+          <t>C1 AI / LLM gateway</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Post 6 (C5, Week 3 Thursday). **Bridge:** Tuesday ends on "the embedding version is production configuration"; Thursday extends that to prompts and every other setting that changes outputs.</t>
+          <t>Post 3 (L2, Week 2 Tuesday). **Bridge:** Managed access is only a safe default if you can leave it; the gateway is what makes leaving a configuration change.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Retrieval quality is a two-stage problem, and it is easy to tune only one stage.</t>
+          <t>The most boring component is the one that makes model switching, and exit plans, possible.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Retrieval quality is a two-stage problem, and it is easy to tune only one stage.</t>
+          <t>The most boring component in the AI stack is the one that makes an exit plan real.</t>
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>#InformationRetrieval #RAG</t>
+          <t>#AIGateway #OperationalResilience</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Funnel diagram: "corpus → stage 1 (embed, k = 50–100, measure recall@k) → stage 2 (rerank, measure nDCG@10) → top passages to the model". Below it, a small "version tag" icon on each vector and a two-index migration strip (old index live, new index shadow, regression gate, cut-over). Source: L7 §7.3 and §7.9 step 6.</t>
+          <t>Hub diagram: applications on the left, one "AI traffic gateway" in the centre (routing, fallback, budgets, policy, log; C2, C3, C4 and C6 plugged in), providers on the right, with a dashed "pre-qualified alternative" route and a stopwatch labelled "time to switch: hours". Below: "two independent deployments, fail closed". Source: C1 §C1.3, §C1.9, §C1.13 H1 view.</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>- "Every vendor except OpenAI offers both" (check for a new OpenAI reranker) - Current model versions if any are named in replies</t>
+          <t>- The PS7/26 / PS26/2 effective date (18 March 2027) - Ownership status of Portkey and OpenRouter - Azure APIM AI Gateway tier status</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
@@ -952,24 +952,24 @@
       <c r="Q8" s="4" t="inlineStr"/>
       <c r="R8" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 5</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 4 · visual 08_Graphic/linkedin/P04.png</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D9" s="5">
-        <f>IF($E$1="","",$E$1+16)</f>
+        <f>IF($E$1="","",$E$1+14)</f>
         <v/>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -979,40 +979,40 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>C5 Prompt and configuration management</t>
+          <t>L3 Agent frameworks and orchestration</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Post 5 (L7, Week 3 Tuesday). **Bridge:** If the embedding version is production configuration, so is the prompt, and both need versioning, review and rollback.</t>
+          <t>Post 6 (C2, Week 3 Thursday). **Bridge:** Tuesday decides how much autonomy a process gets; Thursday explains why guardrails cannot make up for a wrong answer to that question.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Embedding versions and prompts are both production configuration, so they need versioning, review and rollback.</t>
+          <t>Most enterprise "agents" should be deterministic workflows with one judgement step.</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>A one-sentence edit to a prompt can change outputs as much as a model upgrade. Few organisations would let a model upgrade ship without review. Many let prompts change in a web console.</t>
+          <t>Most of the enterprise "agents" I would approve are not agents at all. They are deterministic workflows with one judgement step.</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>#LLMOps #ChangeManagement</t>
+          <t>#AgenticAI #WorkflowAutomation</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>A "release manifest" card for the worked example (illustrative values): prompt set version, drafting model pinned to a dated version, fallback model, embedding and reranker versions, top-k, read-only tool list, guardrail policy version, eval threshold set. Arrows show pull request → second approver → eval gate → tagged release → registry label → trace stamped with version. Source: C5 §C5.12.</t>
+          <t>The worked example's L3 graph as a flow: authorise → fetch attribution snapshot (read-only) → retrieve style and prior commentary → one LLM drafting step → evaluation gate → human approval interrupt → release service. Mark "autonomy budget = 1" on the drafting node and show the checkpoint store beneath the graph. Side panel: three stacked concerns (workflow orchestration, bounded agent steps, durable execution). Source: L3 §3.12 and §3.13.</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>- LaunchDarkly product name (AgentControl) - Langfuse and Promptfoo ownership status</t>
+          <t>- Framework GA and version status; the Agent Builder shutdown date if posting near it - CP4-9 tier statements if any SDK reaches 1.0</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
@@ -1029,24 +1029,24 @@
       <c r="Q9" s="4" t="inlineStr"/>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 6</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 5 · visual 08_Graphic/linkedin/P05.png</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D10" s="5">
-        <f>IF($E$1="","",$E$1+21)</f>
+        <f>IF($E$1="","",$E$1+16)</f>
         <v/>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1056,40 +1056,40 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>L6 Retrieval and knowledge stores</t>
+          <t>C2 Guardrails</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Post 8 (C7, Week 4 Thursday). **Bridge:** Tuesday is about retrieving the right passages under real permissions; Thursday is about the passages someone else wrote for you.</t>
+          <t>Post 5 (L3, Week 3 Tuesday). **Bridge:** Tuesday's deterministic design does most of the safety work; guardrails are the second line, not a licence for more autonomy.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>You may not need a vector database, but you do need retrieval you can measure.</t>
+          <t>Guardrails cannot fix a workflow that should never have been autonomous.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>You may not need a vector database. You do need retrieval you can measure.</t>
+          <t>Guardrails cannot fix a workflow that should never have been autonomous.</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>244</v>
+        <v>257</v>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>#VectorSearch #RAG</t>
+          <t>#AIGuardrails #ResponsibleAI</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Decision-tree graphic (L6 §6.9): Step 0 non-negotiables (filters inside the search, no unfiltered fallback, rebuild tested) → Step 1 "use what you run" (relational database, search engine, document database, object-store tier) → Step 2 three triggers → Step 3 dedicated engine. A side panel contrasts "filter after ranking + fallback = leakage" with "filter inside search + hard empty result".</t>
+          <t>A three-tier pyramid: deterministic rules (base, widest), small classifiers (middle), model-based judges (narrow top), with "fail closed" running down the side. Beside it, "Step 0: decide autonomy first (L3)" as a gate in front of the pyramid. Inset: the worked example's inline numeric-grounding guard. Source: C2 §C2.9 and §C2.12.</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>- pgvector version and any new CVEs - Pinecone Nexus and Weaviate licence status</t>
+          <t>- NeMo Guardrails version; any new Meta guardrail releases - Preview or GA status of Azure Task Adherence</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr">
@@ -1106,24 +1106,24 @@
       <c r="Q10" s="4" t="inlineStr"/>
       <c r="R10" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 7</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 6 · visual 08_Graphic/linkedin/P06.png</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D11" s="5">
-        <f>IF($E$1="","",$E$1+23)</f>
+        <f>IF($E$1="","",$E$1+21)</f>
         <v/>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1133,40 +1133,40 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>C7 AI security</t>
+          <t>L4 Tools, protocols and agent connectivity</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Post 7 (L6, Week 4 Tuesday). **Bridge:** Retrieval brings back passages; some were written by someone who wants your agent to act on them.</t>
+          <t>Post 8 (C4, Week 4 Thursday). **Bridge:** Tuesday puts a gateway in front of every tool; Thursday decides who is allowed through it, and on whose behalf.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Every retrieved document is untrusted input. Indirect prompt injection is a supply-chain problem.</t>
+          <t>Open tool protocols made connecting tools easy, and that is exactly why tool governance now matters.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>A language model follows instructions it finds in any text it reads. Give it tools, and those instructions become actions.</t>
+          <t>Open tool protocols have made it easy to connect an agent to almost anything. That is exactly why tool governance now matters.</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>263</v>
+        <v>242</v>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>#AISecurity #PromptInjection</t>
+          <t>#AgenticAI #APISecurity</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Venn diagram with three circles: untrusted input, sensitive data, outbound channel. The centre is marked "never in one agent". Around it, a defence-in-depth ring for the worked example: deterministic workflow, numeric check, data marking, chunk screening, canary documents, human approval. Source: C7 §C7.9 step 0 and §C7.12.</t>
+          <t>Layer diagram: agent workflow (L3) → tool-governance sub-layer (gateway, private registry, hash-pinned definitions, policy decision, audit) → tools. Tools are colour-coded read-only (green) versus write (amber, "separate approval"). Callout: "45 servers · 20 models · 36.5% average attack success" with the source. Source: L4 §4.2, §4.9 step 0, §4.13 H3 view.</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>- Any new findings on the March 2026 package compromise (intrusion vector is reported two ways) - Acquisition statuses in the security list</t>
+          <t>- Whether a newer MCP specification makes authorisation mandatory - AAIF governance status of MCP and A2A - MCPTox figures (cite the paper directly if challenged)</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
@@ -1183,24 +1183,24 @@
       <c r="Q11" s="4" t="inlineStr"/>
       <c r="R11" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 8</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 7 · visual 08_Graphic/linkedin/P07.png</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D12" s="5">
-        <f>IF($E$1="","",$E$1+28)</f>
+        <f>IF($E$1="","",$E$1+23)</f>
         <v/>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1210,40 +1210,40 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>L4 Tools, protocols and agent connectivity</t>
+          <t>C4 Identity and access for agents</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Post 10 (C4, Week 5 Thursday). **Bridge:** Tuesday puts a gateway in front of every tool; Thursday decides who is allowed through it, and on whose behalf.</t>
+          <t>Post 7 (L4, Week 4 Tuesday). **Bridge:** Once every tool sits behind a gateway, the question is who the agent is, and whose authority it carries.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Open tool protocols made connecting tools easy, and that is exactly why tool governance now matters.</t>
+          <t>"Who did this?" needs an answer when the actor is an agent.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Open tool protocols have made it easy to connect an agent to almost anything. That is exactly why tool governance now matters.</t>
+          <t>"Who did this?" is the first question in every incident review. When the actor is an agent, many logs can answer only with the name of a shared service account.</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>#AgenticAI #APISecurity</t>
+          <t>#IAM #AgenticAI</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Layer diagram: agent workflow (L3) → tool-governance sub-layer (gateway, private registry, hash-pinned definitions, policy decision, audit) → tools. Tools are colour-coded read-only (green) versus write (amber, "separate approval"). Callout: "45 servers · 20 models · 36.5% average attack success" with the source. Source: L4 §4.2, §4.9 step 0, §4.13 H3 view.</t>
+          <t>"One attribution chain" graphic: analyst signs in → token exchange (on behalf of analyst, read-only scope, minutes TTL) → agent identity (sponsor named) → gateway policy decision → tool → audit event (user · agent · tool · args hash · decision · trace ID) → evidence pack. A separate lane shows the approver (different person, step-up authentication). Source: C4 §C4.12.</t>
         </is>
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>- Whether a newer MCP specification makes authorisation mandatory - AAIF governance status of MCP and A2A - MCPTox figures (cite the paper directly if challenged)</t>
+          <t>- Product names and GA status for Entra Agent ID and Okta Agent SSO - Whether any UK or EU rule now names accountability for AI agents</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
@@ -1260,24 +1260,24 @@
       <c r="Q12" s="4" t="inlineStr"/>
       <c r="R12" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 9</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 8 · visual 08_Graphic/linkedin/P08.png</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>5</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D13" s="5">
-        <f>IF($E$1="","",$E$1+30)</f>
+        <f>IF($E$1="","",$E$1+28)</f>
         <v/>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1287,40 +1287,40 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>C4 Identity and access for agents</t>
+          <t>L5 Memory</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Post 9 (L4, Week 5 Tuesday). **Bridge:** Once every tool sits behind a gateway, the question is who the agent is, and whose authority it carries.</t>
+          <t>Post 10 (Regulated reality, Week 5 Thursday). **Bridge:** Memory is where governance gets personal (erasure, retention, reproducibility); Thursday steps back to the regulations that frame all of it.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>"Who did this?" needs an answer when the actor is an agent.</t>
+          <t>What an agent remembers is a governance question before it is a technical one, which is why memory comes last.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>"Who did this?" is the first question in every incident review. When the actor is an agent, many logs can answer only with the name of a shared service account.</t>
+          <t>Memory is the layer I would build last, on purpose. What an agent remembers is a governance question before it is a technical one, and it is the layer I would build last.</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>#IAM #AgenticAI</t>
+          <t>#AgentMemory #DataProtection</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>"One attribution chain" graphic: analyst signs in → token exchange (on behalf of analyst, read-only scope, minutes TTL) → agent identity (sponsor named) → gateway policy decision → tool → audit event (user · agent · tool · args hash · decision · trace ID) → evidence pack. A separate lane shows the approver (different person, step-up authentication). Source: C4 §C4.12.</t>
+          <t>The build-order roadmap (plan §12.6) as a horizontal timeline: governance → evaluation and observability → model access (gateway first) → retrieval → workflows → tools → **memory** (highlighted) → optimisation. Inset: a memory write path with a policy gate (DLP screen, allow-list, approval), a subject index and a "forget-by-subject" arrow reaching store, vectors, revisions and backups. Source: L5 §5.9 and §5.12.</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>- Product names and GA status for Entra Agent ID and Okta Agent SSO - Whether any UK or EU rule now names accountability for AI agents</t>
+          <t>- ICO guidance (under review following the Data (Use and Access) Act) - Memory product defaults (TTL and pruning) and LangMem release status</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr">
@@ -1337,24 +1337,24 @@
       <c r="Q13" s="4" t="inlineStr"/>
       <c r="R13" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 10</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 9 · visual 08_Graphic/linkedin/P09.png</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D14" s="5">
-        <f>IF($E$1="","",$E$1+35)</f>
+        <f>IF($E$1="","",$E$1+30)</f>
         <v/>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1364,40 +1364,40 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>L3 Agent frameworks and orchestration</t>
+          <t>Regulated reality: EU AI Act and DORA</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Post 12 (C2, Week 6 Thursday). **Bridge:** Tuesday decides how much autonomy a process gets; Thursday explains why guardrails cannot make up for a wrong answer to that question.</t>
+          <t>Post 9 (L5, Week 5 Tuesday). **Bridge:** Halfway through the layers, the regulatory frame explains why multi-vendor design and retained evidence stop being optional.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Most enterprise "agents" should be deterministic workflows with one judgement step.</t>
+          <t>Concentration risk turns multi-vendor from a preference into a requirement.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Most of the enterprise "agents" I would approve are not agents at all. They are deterministic workflows with one judgement step.</t>
+          <t>Concentration risk is turning multi-vendor AI from a preference into something close to a requirement.</t>
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>#AgenticAI #WorkflowAutomation</t>
+          <t>#EUAIAct #DORA</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>The worked example's L3 graph as a flow: authorise → fetch attribution snapshot (read-only) → retrieve style and prior commentary → one LLM drafting step → evaluation gate → human approval interrupt → release service. Mark "autonomy budget = 1" on the drafting node and show the checkpoint store beneath the graph. Side panel: three stacked concerns (workflow orchestration, bounded agent steps, durable execution). Source: L3 §3.12 and §3.13.</t>
+          <t>A timeline from April 2026 to December 2027: 17 Apr 2026 SR 26-2 (GenAI out of scope); 13 Jul 2026 UK CTP designations in force; 2 Aug 2026 GPAI enforcement and Article 50 transparency; 18 Mar 2027 UK material third-party notifications; 2 Dec 2027 EU AI Act Annex III. Beneath it, a two-column panel: "designated for direct oversight: hyperscalers and infrastructure" versus "not designated: model vendors (oversight rests on the firm)". Source: regulatory_facts.json and C8 §C8.11.</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>- Framework GA and version status; the Agent Builder shutdown date if posting near it - CP4-9 tier statements if any SDK reaches 1.0</t>
+          <t>- Any update to the DORA CTPP list or new UK CTP designations (especially any model vendor) - Whether the US agencies' AI request for information has been published - EU AI Act dates (any further Omnibus changes) and the PS7/26 effective date - "For most asset-management uses, today's live duties are literacy and transparency" is a judgement; keep it phrased as such</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
@@ -1414,24 +1414,24 @@
       <c r="Q14" s="4" t="inlineStr"/>
       <c r="R14" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 11</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 10 · visual 08_Graphic/linkedin/P10.png</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D15" s="5">
-        <f>IF($E$1="","",$E$1+37)</f>
+        <f>IF($E$1="","",$E$1+35)</f>
         <v/>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1441,40 +1441,40 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>C2 Guardrails</t>
+          <t>L6 Retrieval and knowledge stores</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Post 11 (L3, Week 6 Tuesday). **Bridge:** Tuesday's deterministic design does most of the safety work; guardrails are the second line, not a licence for more autonomy.</t>
+          <t>Post 12 (C7, Week 6 Thursday). **Bridge:** Tuesday is about retrieving the right passages under real permissions; Thursday is about the passages someone else wrote for you.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Guardrails cannot fix a workflow that should never have been autonomous.</t>
+          <t>You may not need a vector database, but you do need retrieval you can measure.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Guardrails cannot fix a workflow that should never have been autonomous.</t>
+          <t>You may not need a vector database. You do need retrieval you can measure.</t>
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>#AIGuardrails #ResponsibleAI</t>
+          <t>#VectorSearch #RAG</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>A three-tier pyramid: deterministic rules (base, widest), small classifiers (middle), model-based judges (narrow top), with "fail closed" running down the side. Beside it, "Step 0: decide autonomy first (L3)" as a gate in front of the pyramid. Inset: the worked example's inline numeric-grounding guard. Source: C2 §C2.9 and §C2.12.</t>
+          <t>Decision-tree graphic (L6 §6.9): Step 0 non-negotiables (filters inside the search, no unfiltered fallback, rebuild tested) → Step 1 "use what you run" (relational database, search engine, document database, object-store tier) → Step 2 three triggers → Step 3 dedicated engine. A side panel contrasts "filter after ranking + fallback = leakage" with "filter inside search + hard empty result".</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>- NeMo Guardrails version; any new Meta guardrail releases - Preview or GA status of Azure Task Adherence</t>
+          <t>- pgvector version and any new CVEs - Pinecone Nexus and Weaviate licence status</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
@@ -1491,24 +1491,24 @@
       <c r="Q15" s="4" t="inlineStr"/>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 12</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 11 · visual 08_Graphic/linkedin/P11.png</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B16" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D16" s="5">
-        <f>IF($E$1="","",$E$1+42)</f>
+        <f>IF($E$1="","",$E$1+37)</f>
         <v/>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1518,40 +1518,40 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>L2 Inference, serving and model access</t>
+          <t>C7 AI security</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Post 14 (C1, Week 7 Thursday). **Bridge:** Tuesday makes managed access the default; Thursday shows the gateway is what keeps that choice reversible.</t>
+          <t>Post 11 (L6, Week 6 Tuesday). **Bridge:** Retrieval brings back passages; some were written by someone who wants your agent to act on them.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Self-hosting is a capacity and operating-model decision, not just a cost decision.</t>
+          <t>Every retrieved document is untrusted input. Indirect prompt injection is a supply-chain problem.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Self-hosting a model is a capacity and operating-model decision. It is only partly a cost decision.</t>
+          <t>A language model follows instructions it finds in any text it reads. Give it tools, and those instructions become actions.</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>#LLMInference #MLOps</t>
+          <t>#AISecurity #PromptInjection</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>L2 split into three stacked sub-layers (serving engines; optimisation, marked "only if you run GPU fleets"; model access), with the gateway lifted out into the control plane. Beside it, a month-end demand curve against a reserved-capacity line, showing headroom and an "overflow stays in region" arrow. Source: L2 §2.3, §2.9 step 3, §2.13 H1 view.</t>
+          <t>Venn diagram with three circles: untrusted input, sensitive data, outbound channel. The centre is marked "never in one agent". Around it, a defence-in-depth ring for the worked example: deterministic workflow, numeric check, data marking, chunk screening, canary documents, human approval. Source: C7 §C7.9 step 0 and §C7.12.</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>- Overflow and residency behaviour statements for each hyperscaler - OpenRouter–Stripe closing; SGLang advisory status</t>
+          <t>- Any new findings on the March 2026 package compromise (intrusion vector is reported two ways) - Acquisition statuses in the security list</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr">
@@ -1568,24 +1568,24 @@
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 13</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 12 · visual 08_Graphic/linkedin/P12.png</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>7</v>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D17" s="5">
-        <f>IF($E$1="","",$E$1+44)</f>
+        <f>IF($E$1="","",$E$1+42)</f>
         <v/>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1595,40 +1595,40 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>C1 AI / LLM gateway</t>
+          <t>L7 Embeddings and reranking</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Post 13 (L2, Week 7 Tuesday). **Bridge:** Managed access is only a safe default if you can leave it; the gateway is what makes leaving a configuration change.</t>
+          <t>Post 14 (C5, Week 7 Thursday). **Bridge:** Tuesday ends on "the embedding version is production configuration"; Thursday extends that to prompts and every other setting that changes outputs.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>The most boring component is the one that makes model switching, and exit plans, possible.</t>
+          <t>Retrieval quality is a two-stage problem, and it is easy to tune only one stage.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>The most boring component in the AI stack is the one that makes an exit plan real.</t>
+          <t>Retrieval quality is a two-stage problem, and it is easy to tune only one stage.</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>#AIGateway #OperationalResilience</t>
+          <t>#InformationRetrieval #RAG</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Hub diagram: applications on the left, one "AI traffic gateway" in the centre (routing, fallback, budgets, policy, log; C2, C3, C4 and C6 plugged in), providers on the right, with a dashed "pre-qualified alternative" route and a stopwatch labelled "time to switch: hours". Below: "two independent deployments, fail closed". Source: C1 §C1.3, §C1.9, §C1.13 H1 view.</t>
+          <t>Funnel diagram: "corpus → stage 1 (embed, k = 50–100, measure recall@k) → stage 2 (rerank, measure nDCG@10) → top passages to the model". Below it, a small "version tag" icon on each vector and a two-index migration strip (old index live, new index shadow, regression gate, cut-over). Source: L7 §7.3 and §7.9 step 6.</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>- The PS7/26 / PS26/2 effective date (18 March 2027) - Ownership status of Portkey and OpenRouter - Azure APIM AI Gateway tier status</t>
+          <t>- "Every vendor except OpenAI offers both" (check for a new OpenAI reranker) - Current model versions if any are named in replies</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
@@ -1645,24 +1645,24 @@
       <c r="Q17" s="4" t="inlineStr"/>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 14</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 13 · visual 08_Graphic/linkedin/P13.png</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D18" s="5">
-        <f>IF($E$1="","",$E$1+49)</f>
+        <f>IF($E$1="","",$E$1+44)</f>
         <v/>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1672,40 +1672,40 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>L1 Foundation models</t>
+          <t>C5 Prompt and configuration management</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Post 16 (C6, Week 8 Thursday). **Bridge:** A portfolio of models needs a way to choose between them on cost without fooling yourself; Thursday supplies the metric.</t>
+          <t>Post 13 (L7, Week 7 Tuesday). **Bridge:** If the embedding version is production configuration, so is the prompt, and both need versioning, review and rollback.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Treat models as a portfolio, not a bet.</t>
+          <t>Embedding versions and prompts are both production configuration, so they need versioning, review and rollback.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Treat foundation models as a portfolio, not a bet.</t>
+          <t>A one-sentence edit to a prompt can change outputs as much as a model upgrade. Few organisations would let a model upgrade ship without review. Many let prompts change in a web console.</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>#FoundationModels #VendorRisk</t>
+          <t>#LLMOps #ChangeManagement</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Portfolio grid: four roles (primary mid tier, fallback mid tier from a different vendor, small classifier, self-hosted open weight) as rows, with columns "pinned version", "region", "qualified on eval suite (date)", "retirement runway". All rows feed one gateway. A "frontier tier: off by default" tile sits above. Source: L1 §1.9 and §1.12 (shown without vendor names).</t>
+          <t>A "release manifest" card for the worked example (illustrative values): prompt set version, drafting model pinned to a dated version, fallback model, embedding and reranker versions, top-k, read-only tool list, guardrail policy version, eval threshold set. Arrows show pull request → second approver → eval gate → tagged release → registry label → trace stamped with version. Source: C5 §C5.12.</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>- The Gemini Flash retirement date and the Claude Fable 5 suspension dates (both cited in the first comment) - Current model families and versions, which change monthly - CP4 tier decisions as published in the final document</t>
+          <t>- LaunchDarkly product name (AgentControl) - Langfuse and Promptfoo ownership status</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
@@ -1722,24 +1722,24 @@
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 15</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 14 · visual 08_Graphic/linkedin/P14.png</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D19" s="5">
-        <f>IF($E$1="","",$E$1+51)</f>
+        <f>IF($E$1="","",$E$1+49)</f>
         <v/>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1749,40 +1749,40 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>C6 AI FinOps</t>
+          <t>L8 Data extraction and ingestion</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Post 15 (L1, Week 8 Tuesday). **Bridge:** A model portfolio is only as good as the cost metric used to choose within it, and cost per token is the wrong one.</t>
+          <t>Post 16 (C3, Week 8 Thursday). **Bridge:** Tuesday shows that quality is decided at ingestion; Thursday shows that residency and privacy are decided there too.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Cost per task, not cost per token, is the metric executives understand.</t>
+          <t>Some of the most convincing "hallucinations" in enterprise retrieval start in a PDF table parser, not in the model.</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Cost per token is the number on the price list. Cost per task is the number executives understand, and the one that tells you whether a change saved anything.</t>
+          <t>Some of the most convincing "hallucinations" in enterprise retrieval systems are not the model's fault. They start in a table parser.</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>262</v>
+        <v>236</v>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>#FinOps #UnitEconomics</t>
+          <t>#RAG #DataQuality</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Side-by-side bars for one approved commentary (illustrative): "token cost" (small) versus "reviewer time" (large), with a third bar "regenerations" that multiplies the token cost. Beneath, the data flow: gateway meter (tags: use case, fund, run ID) → join to trace → monthly reconciliation to invoice → firm-owned cost dataset. Label clearly as illustrative. Source: C6 §C6.9 and §C6.12.</t>
+          <t>Pipeline diagram: source register → acquisition → classification/DLP → parser (drawn as a swappable cartridge) → "metadata envelope" stamped on each chunk (source, version, ACL, classification, parser manifest, lineage ID) → index gate ("no envelope, no index"). A red side-path shows "parsed numbers = context only"; a green path shows "authoritative figures via read-only tool". Source: L8 §8.9 and the six-component control plane in §8.13.</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>- List prices used in the illustrative arithmetic (they change often; "well under a dollar" should still hold) - FOCUS 1.5 ratification status</t>
+          <t>- "Ten products assessed; only one carries ACL metadata; none emits lineage" (check for new lineage features) - Mistral OCR and Docling version status if mentioned in replies</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
@@ -1799,24 +1799,24 @@
       <c r="Q19" s="4" t="inlineStr"/>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 16</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 15 · visual 08_Graphic/linkedin/P15.png</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D20" s="5">
-        <f>IF($E$1="","",$E$1+56)</f>
+        <f>IF($E$1="","",$E$1+51)</f>
         <v/>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -1826,40 +1826,40 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>L5 Memory (deliberately last)</t>
+          <t>C3 DLP and PII protection</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Post 18 (Regulated reality, Week 9 Thursday). **Bridge:** Memory is where governance gets personal (erasure, retention, reproducibility); Thursday steps back to the regulations that frame all of it.</t>
+          <t>Post 15 (L8, Week 8 Tuesday). **Bridge:** If quality is decided at ingestion, so are residency and privacy; a filter at the prompt arrives too late.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>What an agent remembers is a governance question before it is a technical one, which is why memory comes last.</t>
+          <t>Data residency and PII decisions are made at ingestion, not at the prompt.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>I left memory until week nine on purpose. What an agent remembers is a governance question before it is a technical one, and it is the layer I would build last.</t>
+          <t>One analyst question can place the same client identifier in seven places: a prompt, a retrieved chunk, a tool result, a provider's processing region, a trace store, an evaluation dataset and a memory record.</t>
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>#AgentMemory #DataProtection</t>
+          <t>#DataProtection #PrivacyEngineering</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>The build-order roadmap (plan §12.6) as a horizontal timeline: governance → evaluation and observability → model access (gateway first) → retrieval → workflows → tools → **memory** (highlighted) → optimisation. Inset: a memory write path with a policy gate (DLP screen, allow-list, approval), a subject index and a "forget-by-subject" arrow reaching store, vectors, revisions and backups. Source: L5 §5.9 and §5.12.</t>
+          <t>"Seven copies" diagram: one client identifier at the centre with arrows to seven stores (prompt, chunk, tool result, provider region, trace store, eval set, memory). Overlay six numbered enforcement points (E1 ingestion to E6 trace export) all calling one "privacy service" box. Inset: a draft showing CLIENT_A / MANDATE_1 placeholders instead of names. Source: C3 §C3.2, §C3.9 step 0, §C3.12.</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>- ICO guidance (under review following the Data (Use and Access) Act) - Memory product defaults (TTL and pruning) and LangMem release status</t>
+          <t>- Status of the DPF appeal C-703/25 P - Presidio governance and licence - Purview DSPM licensing statement</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
@@ -1876,24 +1876,24 @@
       <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 17</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 16 · visual 08_Graphic/linkedin/P16.png</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B21" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D21" s="5">
-        <f>IF($E$1="","",$E$1+58)</f>
+        <f>IF($E$1="","",$E$1+56)</f>
         <v/>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1903,40 +1903,40 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Regulated reality: EU AI Act and DORA</t>
+          <t>L9 Evaluation and observability</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Post 17 (L5, Week 9 Tuesday). **Bridge:** After eight weeks of layers and controls, the regulatory frame explains why multi-vendor design and retained evidence stop being optional.</t>
+          <t>Post 18 (C8, Week 9 Thursday). **Bridge:** Tuesday argues that evaluation must exist from day one; Thursday shows that the same eval suite, run independently and kept, is the validation evidence a model-risk function needs.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Concentration risk turns multi-vendor from a preference into a requirement.</t>
+          <t>The layer that ages slowest is the one most teams build last, and evals added after go-live measure the damage, not the quality.</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Concentration risk is turning multi-vendor AI from a preference into something close to a requirement.</t>
+          <t>Most diagrams of the AI stack put evaluation in the last box. It is the layer that ages slowest — and the one most teams build last.</t>
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>#EUAIAct #DORA</t>
+          <t>#AIEvaluation #LLMOps</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>A timeline from April 2026 to December 2027: 17 Apr 2026 SR 26-2 (GenAI out of scope); 13 Jul 2026 UK CTP designations in force; 2 Aug 2026 GPAI enforcement and Article 50 transparency; 18 Mar 2027 UK material third-party notifications; 2 Dec 2027 EU AI Act Annex III. Beneath it, a two-column panel: "designated for direct oversight: hyperscalers and infrastructure" versus "not designated: model vendors (oversight rests on the firm)". Source: regulatory_facts.json and C8 §C8.11.</t>
+          <t>Two-panel diagram. Left: the popular nine-layer stack diagram with "Evals and observability" as the last box. Right: the same stack with evaluation and observability redrawn as a vertical plane running alongside every layer, labelled "firm-owned telemetry and evidence spine", with products drawn as replaceable plug-ins. A small callout shows the one metric: "Numeric faithfulness: 100%, any miss blocks." Source: L9 §9.13 and the H8 provisional view.</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>- Any update to the DORA CTPP list or new UK CTP designations (especially any model vendor) - Whether the US agencies' AI request for information has been published - EU AI Act dates (any further Omnibus changes) and the PS7/26 effective date - "For most asset-management uses, today's live duties are literacy and transparency" is a judgement; keep it phrased as such</t>
+          <t>- Arize/Dynatrace completion and the Langfuse/ClickHouse status - Whether OpenAI's Promptfoo acquisition has closed - OpenTelemetry GenAI conventions still at "Development" - The "five of the eleven" count, against the final L9 table</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr">
@@ -1953,24 +1953,24 @@
       <c r="Q21" s="4" t="inlineStr"/>
       <c r="R21" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 18</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 17 · visual 08_Graphic/linkedin/P17.png</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B22" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D22" s="5">
-        <f>IF($E$1="","",$E$1+63)</f>
+        <f>IF($E$1="","",$E$1+58)</f>
         <v/>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1980,40 +1980,40 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>The worked example, end to end</t>
+          <t>C8 Model risk, governance and audit</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Post 20 (Start small, Week 10 Thursday). **Bridge:** Tuesday shows the full worked example and its "never" list; Thursday shows the minimum platform needed to run it, and what to leave out.</t>
+          <t>Post 17 (L9, Week 9 Tuesday). **Bridge:** Tuesday's eval suite becomes Thursday's validation evidence, but only if someone independent challenges it, it is versioned, and it is retained.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>What the attribution-commentary agent must never do matters more than what it can do.</t>
+          <t>Your eval suite *is* your validation evidence. What model-risk discipline means when the "model" is an agent and the main US guidance has stepped aside.</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>For nine weeks one example has run underneath this series: an agent that drafts the monthly performance-attribution commentary for a multi-asset fund, with a portfolio manager approving every draft. It is generic and illustrative. Here it is in one place.</t>
+          <t>In April, the US supervisory guidance that had shaped model risk management since 2011 was replaced. Its successor, SR 26-2, places generative and agentic AI expressly outside its scope.</t>
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>#AgenticAI #AIGovernance</t>
+          <t>#ModelRisk #AIGovernance</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Two-column "may / must never" table for the worked example. Each "never" row has its enforcing component in a coloured chip (read-only tool, numeric comparator, approval interrupt, allow-list, tokenisation, entitlement filter, version pin). Beneath it, the eight-tile evidence pack keyed to one trace ID. Source: synthesis VI.3 and VI.4. Label: "generic, illustrative".</t>
+          <t>One-page "evidence pack" graphic for the worked example: eight tiles (prompt version, model version, data snapshot, tool calls, eval results, approver identity, timestamps, final output), all keyed to one trace ID and feeding an immutable archive. A side panel shows "governed unit = use case" with the model as a vendor component. Source: C8 §C8.12.</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>- No product or regulatory facts in the body. Check that the first comment's per-cloud examples match the final document.</t>
+          <t>- SR 26-2 status, and whether the agencies' AI/GenAI request for information has been published (update the post if it has) - SS1/23 scope statements - Collibra–trail ML completion</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
@@ -2030,24 +2030,24 @@
       <c r="Q22" s="4" t="inlineStr"/>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 19</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 18 · visual 08_Graphic/linkedin/P18.png</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B23" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D23" s="5">
-        <f>IF($E$1="","",$E$1+65)</f>
+        <f>IF($E$1="","",$E$1+63)</f>
         <v/>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -2057,40 +2057,40 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Start small</t>
+          <t>The worked example, end to end</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Post 19 (Worked example, Week 10 Tuesday). **Bridge:** Tuesday's agent needs a platform; Thursday argues that the minimum platform, plus a published "not yet" list, is the right first release.</t>
+          <t>Post 20 (Start small, Week 10 Thursday). **Bridge:** Tuesday shows the full worked example and its "never" list; Thursday shows the minimum platform needed to run it, and what to leave out.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>The most valuable part of a reference architecture is the "do not build yet" list.</t>
+          <t>What the attribution-commentary agent must never do matters more than what it can do.</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>The most valuable page in a reference architecture is often the "do not build yet" list.</t>
+          <t>For nine weeks one example has run underneath this series: an agent that drafts the monthly performance-attribution commentary for a multi-asset fund, with a portfolio manager approving every draft. It is generic and illustrative. Here it is in one place.</t>
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>#EnterpriseArchitecture #AgenticAI</t>
+          <t>#AgenticAI #AIGovernance</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Two panels. Left, "Build now": the Stack D minimum as a compact stack (gateway ×2, identity, manifest, checks, eval suite, one store, one workflow, two models). Right, "Do NOT build yet": the not-yet items as greyed-out tiles, each with a one-word trigger for revisiting it ("evidence", "load test", "use case"). Source: synthesis Part VII, Stack D.</t>
+          <t>Two-column "may / must never" table for the worked example. Each "never" row has its enforcing component in a coloured chip (read-only tool, numeric comparator, approval interrupt, allow-list, tokenisation, entitlement filter, version pin). Beneath it, the eight-tile evidence pack keyed to one trace ID. Source: synthesis VI.3 and VI.4. Label: "generic, illustrative".</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>- The not-yet list against the final Part VII and the Part XI tiers (anything promoted from Experimental)</t>
+          <t>- No product or regulatory facts in the body. Check that the first comment's per-cloud examples match the final document.</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
@@ -2107,24 +2107,24 @@
       <c r="Q23" s="4" t="inlineStr"/>
       <c r="R23" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 20</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 19 · visual 08_Graphic/linkedin/P19.png</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B24" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D24" s="5">
-        <f>IF($E$1="","",$E$1+70)</f>
+        <f>IF($E$1="","",$E$1+65)</f>
         <v/>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -2134,40 +2134,40 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Build vs buy</t>
+          <t>Start small</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Post 22 (Where not to abstract, Week 11 Thursday). **Bridge:** Tuesday says to own a thin interface in front of what you buy; Thursday warns against owning too many interfaces.</t>
+          <t>Post 19 (Worked example, Week 10 Tuesday). **Bridge:** Tuesday's agent needs a platform; Thursday argues that the minimum platform, plus a published "not yet" list, is the right first release.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Build where you differentiate, buy where you would only be maintaining.</t>
+          <t>The most valuable part of a reference architecture is the "do not build yet" list.</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Build where you differentiate. Buy where you would only be maintaining.</t>
+          <t>The most valuable page in a reference architecture is often the "do not build yet" list.</t>
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>#EnterpriseArchitecture #BuildVsBuy</t>
+          <t>#EnterpriseArchitecture #AgenticAI</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>Three-column board, "Build · Hybrid · Buy", with the 17 layers and controls placed as cards (for example, Build: tool servers, configuration of record, evidence store; Hybrid: gateway, guardrails, privacy, evaluation, retrieval optimisation; Buy: security tooling, foundation models, serving access). A separate red card reads "Do not build yet: fine-tuning". Source: synthesis Part VIII table.</t>
+          <t>Two panels. Left, "Build now": the Stack D minimum as a compact stack (gateway ×2, identity, manifest, checks, eval suite, one store, one workflow, two models). Right, "Do NOT build yet": the not-yet items as greyed-out tiles, each with a one-word trigger for revisiting it ("evidence", "load test", "use case"). Source: synthesis Part VII, Stack D.</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>- No dated facts in the body. Check the Article 25 wording if challenged ("can, in some cases").</t>
+          <t>- The not-yet list against the final Part VII and the Part XI tiers (anything promoted from Experimental)</t>
         </is>
       </c>
       <c r="N24" s="4" t="inlineStr">
@@ -2184,24 +2184,24 @@
       <c r="Q24" s="4" t="inlineStr"/>
       <c r="R24" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 21</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 20 · visual 08_Graphic/linkedin/P20.png</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B25" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D25" s="5">
-        <f>IF($E$1="","",$E$1+72)</f>
+        <f>IF($E$1="","",$E$1+70)</f>
         <v/>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -2211,40 +2211,40 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Where not to abstract</t>
+          <t>Build vs buy</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Post 21 (Build vs buy, Week 11 Tuesday). **Bridge:** Tuesday's thin firm-owned interfaces are the right default; Thursday names where adding one is the mistake.</t>
+          <t>Post 22 (Where not to abstract, Week 11 Thursday). **Bridge:** Tuesday says to own a thin interface in front of what you buy; Thursday warns against owning too many interfaces.</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Frameworks on top of frameworks.</t>
+          <t>Build where you differentiate, buy where you would only be maintaining.</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Abstraction is how an architecture stays reversible. Too much of it is how an architecture stops moving.</t>
+          <t>Build where you differentiate. Buy where you would only be maintaining.</t>
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>#SoftwareArchitecture #AgenticAI</t>
+          <t>#EnterpriseArchitecture #BuildVsBuy</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>Two lists side by side. "Abstract (thin, firm-owned)": routing contract, telemetry collector, datasets, credentials, policy, retrieval interface, embed/rerank, privacy API, memory API, config fetch. "Do not over-abstract": agent frameworks, single-workflow plug-ins, plain database access, store-bundled features, vendor model extras. A small strip beneath shows "multi-vendor necessary" versus "multi-vendor only adds complexity". Source: synthesis IX.1–IX.3.</t>
+          <t>Three-column board, "Build · Hybrid · Buy", with the 17 layers and controls placed as cards (for example, Build: tool servers, configuration of record, evidence store; Hybrid: gateway, guardrails, privacy, evaluation, retrieval optimisation; Buy: security tooling, foundation models, serving access). A separate red card reads "Do not build yet: fine-tuning". Source: synthesis Part VIII table.</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>- No dated facts in the body.</t>
+          <t>- No dated facts in the body. Check the Article 25 wording if challenged ("can, in some cases").</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
@@ -2261,24 +2261,24 @@
       <c r="Q25" s="4" t="inlineStr"/>
       <c r="R25" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 22</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 21 · visual 08_Graphic/linkedin/P21.png</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B26" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="D26" s="5">
-        <f>IF($E$1="","",$E$1+77)</f>
+        <f>IF($E$1="","",$E$1+72)</f>
         <v/>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -2288,40 +2288,40 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Which lock-in is acceptable</t>
+          <t>Where not to abstract</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Post 24 (Close, Week 12 Thursday). **Bridge:** Tuesday classifies which dependencies are worth accepting; Thursday applies that to the final stack: what I would select, and what I would deliberately leave out.</t>
+          <t>Post 21 (Build vs buy, Week 11 Tuesday). **Bridge:** Tuesday's thin firm-owned interfaces are the right default; Thursday names where adding one is the mistake.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Some lock-in is a good trade, and the skill is knowing which.</t>
+          <t>Frameworks on top of frameworks.</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Some lock-in is a good trade. The skill is knowing which.</t>
+          <t>Abstraction is how an architecture stays reversible. Too much of it is how an architecture stops moving.</t>
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>#VendorRisk #EnterpriseArchitecture</t>
+          <t>#SoftwareArchitecture #AgenticAI</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Heat-map table: the 17 layers and controls as rows; columns "acceptable", "manageable", "unacceptable"; each cell a short phrase from the synthesis table (vendor names removed). A highlighted band across the "unacceptable" column reads "the firm's own records: evidence, configuration, datasets, credentials". Source: synthesis IX.4.</t>
+          <t>Two lists side by side. "Abstract (thin, firm-owned)": routing contract, telemetry collector, datasets, credentials, policy, retrieval interface, embed/rerank, privacy API, memory API, config fetch. "Do not over-abstract": agent frameworks, single-workflow plug-ins, plain database access, store-bundled features, vendor model extras. A small strip beneath shows "multi-vendor necessary" versus "multi-vendor only adds complexity". Source: synthesis IX.1–IX.3.</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>- Lock-in categories against the final Part IX.4 table - Any new ownership change in a "manageable" category</t>
+          <t>- No dated facts in the body.</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -2338,24 +2338,24 @@
       <c r="Q26" s="4" t="inlineStr"/>
       <c r="R26" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 23</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 22 · visual 08_Graphic/linkedin/P22.png</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B27" s="4" t="n">
         <v>12</v>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="D27" s="5">
-        <f>IF($E$1="","",$E$1+79)</f>
+        <f>IF($E$1="","",$E$1+77)</f>
         <v/>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -2365,40 +2365,40 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Close: what I'd select, and what I'd deliberately not select</t>
+          <t>Which lock-in is acceptable</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Post 23 (Which lock-in is acceptable, Week 12 Tuesday). **Bridge:** Tuesday's lock-in classification is the filter; Thursday shows what passes through it, what does not, and what leading the change actually requires.</t>
+          <t>Post 24 (Close, Week 12 Thursday). **Bridge:** Tuesday classifies which dependencies are worth accepting; Thursday applies that to the final stack: what I would select, and what I would deliberately leave out.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>The full stack on one page, plus a lesson about leading the transformation.</t>
+          <t>Some lock-in is a good trade, and the skill is knowing which.</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Twelve weeks ago this series started from a popular diagram of the AI stack. On this review, 39 of its 80 product tiles were out of date. The diagram was a catalogue. The enterprise problem is a control system.</t>
+          <t>Some lock-in is a good trade. The skill is knowing which.</t>
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>#EnterpriseArchitecture #AIGovernance</t>
+          <t>#VendorRisk #EnterpriseArchitecture</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>The one-page architecture from synthesis I.2, with vendor names removed: control plane (C1–C8 with the L9 evidence plane) across the top; agent, knowledge and model planes beneath. To the right, a short "Deliberately not selected" column with the categories from XI.5 and XI.7. Optional carousel: slide 1 the original diagram with 39 tiles flagged; slide 2 the one-page architecture; slide 3 the twelve decisions; slide 4 "not selected".</t>
+          <t>Heat-map table: the 17 layers and controls as rows; columns "acceptable", "manageable", "unacceptable"; each cell a short phrase from the synthesis table (vendor names removed). A highlighted band across the "unacceptable" column reads "the firm's own records: evidence, configuration, datasets, credentials". Source: synthesis IX.4.</t>
         </is>
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>- The final Part XI lists (avoid and monitor), especially any item that has changed tier since October 2026 - Ownership and status changes across the products in the first comment</t>
+          <t>- Lock-in categories against the final Part IX.4 table - Any new ownership change in a "manageable" category</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -2415,13 +2415,90 @@
       <c r="Q27" s="4" t="inlineStr"/>
       <c r="R27" s="4" t="inlineStr">
         <is>
-          <t>Master_Architecture: LinkedIn series, Post 24</t>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 23 · visual 08_Graphic/linkedin/P23.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D28" s="5">
+        <f>IF($E$1="","",$E$1+79)</f>
+        <v/>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Close: what I'd select, and what I'd deliberately not select</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Post 23 (Which lock-in is acceptable, Week 12 Tuesday). **Bridge:** Tuesday's lock-in classification is the filter; Thursday shows what passes through it, what does not, and what leading the change actually requires.</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>The full stack on one page, plus a lesson about leading the transformation.</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>Twelve weeks ago this series started from a popular diagram of the AI stack. On this review, 39 of its 80 product tiles were out of date. The diagram was a catalogue. The enterprise problem is a control system.</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>269</v>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>#EnterpriseArchitecture #AIGovernance</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>The one-page architecture from synthesis I.2, with vendor names removed: control plane (C1–C8 with the L9 evidence plane) across the top; agent, knowledge and model planes beneath. To the right, a short "Deliberately not selected" column with the categories from XI.5 and XI.7. Optional carousel: slide 1 the popular stack diagram with 39 tiles flagged; slide 2 the one-page architecture; slide 3 the twelve decisions; slide 4 "not selected".</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>- The final Part XI lists (avoid and monitor), especially any item that has changed tier since October 2026 - Ownership and status changes across the products in the first comment</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="P28" s="4" t="inlineStr"/>
+      <c r="Q28" s="4" t="inlineStr"/>
+      <c r="R28" s="4" t="inlineStr">
+        <is>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 24 · visual 08_Graphic/linkedin/P24.png</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="N4:N27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N4:N28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Draft,Anecdote added,Scheduled,Published,Skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
LinkedIn: no fixed weekday — posts, bridges, visuals and calendar no longer name Tuesday/Thursday (user decision 10 Oct 2026)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYt6k15P64MhHqeyveeQ6D
</commit_message>
<xml_diff>
--- a/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
+++ b/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="ddd dd mmm yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd mmm yyyy"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -469,13 +469,13 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Series start date (first Tuesday after CP5 sign-off):</t>
+          <t>Series start date (the date you publish Post 1):</t>
         </is>
       </c>
       <c r="E1" s="2" t="n"/>
       <c r="F1" t="inlineStr">
         <is>
-          <t>← enter the start Tuesday (dates and times below compute from it; posting time about 08:00 UK)</t>
+          <t>← enter the date of Post 1; suggested dates below compute from it (any weekday; edit freely)</t>
         </is>
       </c>
     </row>
@@ -492,12 +492,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Slot</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Suggested date</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -580,11 +580,11 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Introduction</t>
         </is>
       </c>
       <c r="D4" s="5">
-        <f>IF($E$1="","",$E$1+-5)</f>
+        <f>IF($E$1="","",$E$1+-3)</f>
         <v/>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Post 1 (L1, Week 1 Tuesday). **Bridge:** The series starts where every architecture starts: the models, and how not to bet the firm on one of them.</t>
+          <t>Post 1 (L1, Week 1). **Bridge:** The series starts where every architecture starts: the models, and how not to bet the firm on one of them.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="J4" s="4" t="n">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
@@ -622,12 +622,12 @@
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Series map: the nine layers (L1 → L9) as a stack on the left, each paired by a connector with its Thursday control or theme on the right, labelled with week numbers 1–9. Weeks 10–12 (worked example, start small, build vs buy, where not to abstract, lock-in, close) as a strip beneath. A banner across the top: "the control plane around the products is the architecture". Footer: "24 posts · 12 weeks · one worked example". Source: the calendar above and synthesis Part I.</t>
+          <t>Series map: the nine layers (L1 → L9) as a stack on the left, each paired by a connector with its control or theme on the right, labelled with week numbers 1–9. Weeks 10–12 (worked example, start small, build vs buy, where not to abstract, lock-in, close) as a strip beneath. A banner across the top: "the control plane around the products is the architecture". Footer: "24 posts · 12 weeks · one worked example". Source: the calendar above and synthesis Part I.</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>- The counts (140 products, 1,255 sources, 39 of 80 tiles) against the final published edition - The start date of Post 1 (the first Tuesday after sign-off)</t>
+          <t>- The counts (140 products, 1,255 sources, 39 of 80 tiles) against the final published edition - The planned date of Post 1 (set in the content calendar)</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D5" s="5">
@@ -676,7 +676,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Post 2 (C6, Week 1 Thursday). **Bridge:** A portfolio of models needs a way to choose between them on cost without fooling yourself; Thursday supplies the metric.</t>
+          <t>Post 2 (C6, Week 1). **Bridge:** A portfolio of models needs a way to choose between them on cost without fooling yourself; the control post supplies the metric.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D6" s="5">
@@ -753,7 +753,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Post 1 (L1, Week 1 Tuesday). **Bridge:** A model portfolio is only as good as the cost metric used to choose within it, and cost per token is the wrong one.</t>
+          <t>Post 1 (L1, Week 1). **Bridge:** A model portfolio is only as good as the cost metric used to choose within it, and cost per token is the wrong one.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D7" s="5">
@@ -830,7 +830,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Post 4 (C1, Week 2 Thursday). **Bridge:** Tuesday makes managed access the default; Thursday shows the gateway is what keeps that choice reversible.</t>
+          <t>Post 4 (C1, Week 2). **Bridge:** The stack post makes managed access the default; the control post shows the gateway is what keeps that choice reversible.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D8" s="5">
@@ -907,7 +907,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Post 3 (L2, Week 2 Tuesday). **Bridge:** Managed access is only a safe default if you can leave it; the gateway is what makes leaving a configuration change.</t>
+          <t>Post 3 (L2, Week 2). **Bridge:** Managed access is only a safe default if you can leave it; the gateway is what makes leaving a configuration change.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
@@ -965,7 +965,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D9" s="5">
@@ -984,7 +984,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Post 6 (C2, Week 3 Thursday). **Bridge:** Tuesday decides how much autonomy a process gets; Thursday explains why guardrails cannot make up for a wrong answer to that question.</t>
+          <t>Post 6 (C2, Week 3). **Bridge:** The stack post decides how much autonomy a process gets; the control post explains why guardrails cannot make up for a wrong answer to that question.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D10" s="5">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Post 5 (L3, Week 3 Tuesday). **Bridge:** Tuesday's deterministic design does most of the safety work; guardrails are the second line, not a licence for more autonomy.</t>
+          <t>Post 5 (L3, Week 3). **Bridge:** The stack post's deterministic design does most of the safety work; guardrails are the second line, not a licence for more autonomy.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1075,7 +1075,7 @@
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D11" s="5">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Post 8 (C4, Week 4 Thursday). **Bridge:** Tuesday puts a gateway in front of every tool; Thursday decides who is allowed through it, and on whose behalf.</t>
+          <t>Post 8 (C4, Week 4). **Bridge:** The stack post puts a gateway in front of every tool; the control post decides who is allowed through it, and on whose behalf.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D12" s="5">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Post 7 (L4, Week 4 Tuesday). **Bridge:** Once every tool sits behind a gateway, the question is who the agent is, and whose authority it carries.</t>
+          <t>Post 7 (L4, Week 4). **Bridge:** Once every tool sits behind a gateway, the question is who the agent is, and whose authority it carries.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D13" s="5">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Post 10 (Regulated reality, Week 5 Thursday). **Bridge:** Memory is where governance gets personal (erasure, retention, reproducibility); Thursday steps back to the regulations that frame all of it.</t>
+          <t>Post 10 (Regulated reality, Week 5). **Bridge:** Memory is where governance gets personal (erasure, retention, reproducibility); the control post steps back to the regulations that frame all of it.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D14" s="5">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Post 9 (L5, Week 5 Tuesday). **Bridge:** Halfway through the layers, the regulatory frame explains why multi-vendor design and retained evidence stop being optional.</t>
+          <t>Post 9 (L5, Week 5). **Bridge:** Halfway through the layers, the regulatory frame explains why multi-vendor design and retained evidence stop being optional.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D15" s="5">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Post 12 (C7, Week 6 Thursday). **Bridge:** Tuesday is about retrieving the right passages under real permissions; Thursday is about the passages someone else wrote for you.</t>
+          <t>Post 12 (C7, Week 6). **Bridge:** The stack post is about retrieving the right passages under real permissions; the control post is about the passages someone else wrote for you.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D16" s="5">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Post 11 (L6, Week 6 Tuesday). **Bridge:** Retrieval brings back passages; some were written by someone who wants your agent to act on them.</t>
+          <t>Post 11 (L6, Week 6). **Bridge:** Retrieval brings back passages; some were written by someone who wants your agent to act on them.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D17" s="5">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Post 14 (C5, Week 7 Thursday). **Bridge:** Tuesday ends on "the embedding version is production configuration"; Thursday extends that to prompts and every other setting that changes outputs.</t>
+          <t>Post 14 (C5, Week 7). **Bridge:** The stack post ends on "the embedding version is production configuration"; the control post extends that to prompts and every other setting that changes outputs.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D18" s="5">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Post 13 (L7, Week 7 Tuesday). **Bridge:** If the embedding version is production configuration, so is the prompt, and both need versioning, review and rollback.</t>
+          <t>Post 13 (L7, Week 7). **Bridge:** If the embedding version is production configuration, so is the prompt, and both need versioning, review and rollback.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1691,7 +1691,7 @@
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D19" s="5">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Post 16 (C3, Week 8 Thursday). **Bridge:** Tuesday shows that quality is decided at ingestion; Thursday shows that residency and privacy are decided there too.</t>
+          <t>Post 16 (C3, Week 8). **Bridge:** The stack post shows that quality is decided at ingestion; the control post shows that residency and privacy are decided there too.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D20" s="5">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Post 15 (L8, Week 8 Tuesday). **Bridge:** If quality is decided at ingestion, so are residency and privacy; a filter at the prompt arrives too late.</t>
+          <t>Post 15 (L8, Week 8). **Bridge:** If quality is decided at ingestion, so are residency and privacy; a filter at the prompt arrives too late.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D21" s="5">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Post 18 (C8, Week 9 Thursday). **Bridge:** Tuesday argues that evaluation must exist from day one; Thursday shows that the same eval suite, run independently and kept, is the validation evidence a model-risk function needs.</t>
+          <t>Post 18 (C8, Week 9). **Bridge:** The stack post argues that evaluation must exist from day one; the control post shows that the same eval suite, run independently and kept, is the validation evidence a model-risk function needs.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D22" s="5">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Post 17 (L9, Week 9 Tuesday). **Bridge:** Tuesday's eval suite becomes Thursday's validation evidence, but only if someone independent challenges it, it is versioned, and it is retained.</t>
+          <t>Post 17 (L9, Week 9). **Bridge:** The stack post's eval suite becomes the control post's validation evidence, but only if someone independent challenges it, it is versioned, and it is retained.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1999,7 +1999,7 @@
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D23" s="5">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Post 20 (Start small, Week 10 Thursday). **Bridge:** Tuesday shows the full worked example and its "never" list; Thursday shows the minimum platform needed to run it, and what to leave out.</t>
+          <t>Post 20 (Start small, Week 10). **Bridge:** The stack post shows the full worked example and its "never" list; the control post shows the minimum platform needed to run it, and what to leave out.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D24" s="5">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Post 19 (Worked example, Week 10 Tuesday). **Bridge:** Tuesday's agent needs a platform; Thursday argues that the minimum platform, plus a published "not yet" list, is the right first release.</t>
+          <t>Post 19 (Worked example, Week 10). **Bridge:** The stack post's agent needs a platform; the control post argues that the minimum platform, plus a published "not yet" list, is the right first release.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D25" s="5">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Post 22 (Where not to abstract, Week 11 Thursday). **Bridge:** Tuesday says to own a thin interface in front of what you buy; Thursday warns against owning too many interfaces.</t>
+          <t>Post 22 (Where not to abstract, Week 11). **Bridge:** The stack post says to own a thin interface in front of what you buy; the control post warns against owning too many interfaces.</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D26" s="5">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Post 21 (Build vs buy, Week 11 Tuesday). **Bridge:** Tuesday's thin firm-owned interfaces are the right default; Thursday names where adding one is the mistake.</t>
+          <t>Post 21 (Build vs buy, Week 11). **Bridge:** The stack post's thin firm-owned interfaces are the right default; the control post names where adding one is the mistake.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Stack post</t>
         </is>
       </c>
       <c r="D27" s="5">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Post 24 (Close, Week 12 Thursday). **Bridge:** Tuesday classifies which dependencies are worth accepting; Thursday applies that to the final stack: what I would select, and what I would deliberately leave out.</t>
+          <t>Post 24 (Close, Week 12). **Bridge:** The stack post classifies which dependencies are worth accepting; the control post applies that to the final stack: what I would select, and what I would deliberately leave out.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Control post</t>
         </is>
       </c>
       <c r="D28" s="5">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Post 23 (Which lock-in is acceptable, Week 12 Tuesday). **Bridge:** Tuesday's lock-in classification is the filter; Thursday shows what passes through it, what does not, and what leading the change actually requires.</t>
+          <t>Post 23 (Which lock-in is acceptable, Week 12). **Bridge:** The stack post's lock-in classification is the filter; the control post shows what passes through it, what does not, and what leading the change actually requires.</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Worked example built post by post: worked_example_build.json drives a progress strip on every post visual, a step line in each first comment, a calendar column and an appendix table
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYt6k15P64MhHqeyveeQ6D
</commit_message>
<xml_diff>
--- a/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
+++ b/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R28"/>
+  <dimension ref="A1:S28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -452,18 +452,19 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
     <col width="45" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="25" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="17" max="17"/>
     <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -512,60 +513,65 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
+          <t>Worked example step</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
           <t>Pair</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Tension</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Hook (first line)</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Words</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Hashtags</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Visual brief</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Re-verify before posting</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Cleared</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>Published URL</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>Responses / notes</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>Full post and visual</t>
         </is>
@@ -599,50 +605,55 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
+          <t>The brief: The use case and its boundary: the agent writes words around numbers it is given; it never produces a number, and a named portfolio manager approves every draft.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
           <t>Post 1 (L1, Week 1). **Bridge:** The series starts where every architecture starts: the models, and how not to bet the firm on one of them.</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>The logos move faster than any diagram; the controls around them are what last.</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Over the next twelve weeks I am going to take the enterprise GenAI stack apart, one layer at a time.</t>
         </is>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>233</v>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>#GenerativeAI #EnterpriseArchitecture</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Series map: the nine layers (L1 → L9) as a stack on the left, each paired by a connector with its control or theme on the right, labelled with week numbers 1–9. Weeks 10–12 (worked example, start small, build vs buy, where not to abstract, lock-in, close) as a strip beneath. A banner across the top: "the control plane around the products is the architecture". Footer: "24 posts · 12 weeks · one worked example". Source: the calendar above and synthesis Part I.</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>- The counts (140 products, 1,255 sources, 39 of 80 tiles) against the final published edition - The planned date of Post 1 (set in the content calendar)</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P4" s="4" t="inlineStr"/>
       <c r="Q4" s="4" t="inlineStr"/>
-      <c r="R4" s="4" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr"/>
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 0 · visual 08_Graphic/linkedin/P00.png</t>
         </is>
@@ -676,50 +687,55 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
+          <t>Models: Four model roles, each pinned to an exact version: a primary drafting model, a fallback from a different vendor, a small classifier for reviewer edits, and a self-hosted open-weight model for anything touching unmasked client data.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t>Post 2 (C6, Week 1). **Bridge:** A portfolio of models needs a way to choose between them on cost without fooling yourself; the control post supplies the metric.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Treat models as a portfolio, not a bet.</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Treat foundation models as a portfolio, not a bet.</t>
         </is>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>241</v>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>#FoundationModels #VendorRisk</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Portfolio grid: four roles (primary mid tier, fallback mid tier from a different vendor, small classifier, self-hosted open weight) as rows, with columns "pinned version", "region", "qualified on eval suite (date)", "retirement runway". All rows feed one gateway. A "frontier tier: off by default" tile sits above. Source: L1 §1.9 and §1.12 (shown without vendor names).</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>- The Gemini Flash retirement date and the Claude Fable 5 suspension dates (both cited in the first comment) - Current model families and versions, which change monthly - CP4 tier decisions as published in the final document</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr"/>
       <c r="Q5" s="4" t="inlineStr"/>
-      <c r="R5" s="4" t="inlineStr">
+      <c r="R5" s="4" t="inlineStr"/>
+      <c r="S5" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 1 · visual 08_Graphic/linkedin/P01.png</t>
         </is>
@@ -753,50 +769,55 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
+          <t>Cost: A run ID on every call, tagged with use case and fund, joined to the trace; a monthly budget set from two month-end cycles; a per-run ceiling on model calls and tokens.</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
           <t>Post 1 (L1, Week 1). **Bridge:** A model portfolio is only as good as the cost metric used to choose within it, and cost per token is the wrong one.</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Cost per task, not cost per token, is the metric executives understand.</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>Cost per token is the number on the price list. Cost per task is the number executives understand, and the one that tells you whether a change saved anything.</t>
         </is>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="K6" s="4" t="n">
         <v>263</v>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>#FinOps #UnitEconomics</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>Side-by-side bars for one approved commentary (illustrative): "token cost" (small) versus "reviewer time" (large), with a third bar "regenerations" that multiplies the token cost. Beneath, the data flow: gateway meter (tags: use case, fund, run ID) → join to trace → monthly reconciliation to invoice → firm-owned cost dataset. Label clearly as illustrative. Source: C6 §C6.9 and §C6.12.</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>- List prices used in the illustrative arithmetic (they change often; "well under a dollar" should still hold) - FOCUS 1.5 ratification status</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P6" s="4" t="inlineStr"/>
       <c r="Q6" s="4" t="inlineStr"/>
-      <c r="R6" s="4" t="inlineStr">
+      <c r="R6" s="4" t="inlineStr"/>
+      <c r="S6" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 2 · visual 08_Graphic/linkedin/P02.png</t>
         </is>
@@ -830,50 +851,55 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
+          <t>Model access: Drafting through the primary cloud's in-region model service, with capacity sized for the month-end peak and an open-weight route kept ready as the stressed exit.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
           <t>Post 4 (C1, Week 2). **Bridge:** The stack post makes managed access the default; the control post shows the gateway is what keeps that choice reversible.</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Self-hosting is a capacity and operating-model decision, not just a cost decision.</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>Self-hosting a model is a capacity and operating-model decision. It is only partly a cost decision.</t>
         </is>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>253</v>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>#LLMInference #MLOps</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>L2 split into three stacked sub-layers (serving engines; optimisation, marked "only if you run GPU fleets"; model access), with the gateway lifted out into the control plane. Beside it, a month-end demand curve against a reserved-capacity line, showing headroom and an "overflow stays in region" arrow. Source: L2 §2.3, §2.9 step 3, §2.13 H1 view.</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>- Overflow and residency behaviour statements for each hyperscaler - OpenRouter–Stripe closing; SGLang advisory status</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P7" s="4" t="inlineStr"/>
       <c r="Q7" s="4" t="inlineStr"/>
-      <c r="R7" s="4" t="inlineStr">
+      <c r="R7" s="4" t="inlineStr"/>
+      <c r="S7" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 3 · visual 08_Graphic/linkedin/P03.png</t>
         </is>
@@ -907,50 +933,55 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
+          <t>Gateway: One gateway route, attribution-commentary-draft: the workflow calls the route with its own identity and never holds a provider key; residency, fallback, budgets and inline guards live on the route.</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
           <t>Post 3 (L2, Week 2). **Bridge:** Managed access is only a safe default if you can leave it; the gateway is what makes leaving a configuration change.</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>The most boring component is the one that makes model switching, and exit plans, possible.</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>The most boring component in the AI stack is the one that makes an exit plan real.</t>
         </is>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>253</v>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>#AIGateway #OperationalResilience</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>Hub diagram: applications on the left, one "AI traffic gateway" in the centre (routing, fallback, budgets, policy, log; C2, C3, C4 and C6 plugged in), providers on the right, with a dashed "pre-qualified alternative" route and a stopwatch labelled "time to switch: hours". Below: "two independent deployments, fail closed". Source: C1 §C1.3, §C1.9, §C1.13 H1 view.</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>- The PS7/26 / PS26/2 effective date (18 March 2027) - Ownership status of Portkey and OpenRouter - Azure APIM AI Gateway tier status</t>
         </is>
       </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O8" s="4" t="inlineStr">
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P8" s="4" t="inlineStr"/>
       <c r="Q8" s="4" t="inlineStr"/>
-      <c r="R8" s="4" t="inlineStr">
+      <c r="R8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 4 · visual 08_Graphic/linkedin/P04.png</t>
         </is>
@@ -984,50 +1015,55 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
+          <t>Workflow: A pinned workflow graph: authorise, fetch the attribution snapshot, retrieve style and prior commentary, one drafting step, an evaluation gate, a human approval interrupt, then release by a separate service.</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
           <t>Post 6 (C2, Week 3). **Bridge:** The stack post decides how much autonomy a process gets; the control post explains why guardrails cannot make up for a wrong answer to that question.</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Most enterprise "agents" should be deterministic workflows with one judgement step.</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>Most of the enterprise "agents" I would approve are not agents at all. They are deterministic workflows with one judgement step.</t>
         </is>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="K9" s="4" t="n">
         <v>256</v>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>#AgenticAI #WorkflowAutomation</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>The worked example's L3 graph as a flow: authorise → fetch attribution snapshot (read-only) → retrieve style and prior commentary → one LLM drafting step → evaluation gate → human approval interrupt → release service. Mark "autonomy budget = 1" on the drafting node and show the checkpoint store beneath the graph. Side panel: three stacked concerns (workflow orchestration, bounded agent steps, durable execution). Source: L3 §3.12 and §3.13.</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>- Framework GA and version status; the Agent Builder shutdown date if posting near it - CP4-9 tier statements if any SDK reaches 1.0</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P9" s="4" t="inlineStr"/>
       <c r="Q9" s="4" t="inlineStr"/>
-      <c r="R9" s="4" t="inlineStr">
+      <c r="R9" s="4" t="inlineStr"/>
+      <c r="S9" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 5 · visual 08_Graphic/linkedin/P05.png</t>
         </is>
@@ -1061,50 +1097,55 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
+          <t>Guardrails: A deterministic numeric comparator on every draft, injection screening of retrieved text, a PII check on output and denied topics (forecasts, advice).</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
           <t>Post 5 (L3, Week 3). **Bridge:** The stack post's deterministic design does most of the safety work; guardrails are the second line, not a licence for more autonomy.</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Guardrails cannot fix a workflow that should never have been autonomous.</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>Guardrails cannot fix a workflow that should never have been autonomous.</t>
         </is>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="K10" s="4" t="n">
         <v>258</v>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>#AIGuardrails #ResponsibleAI</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>A three-tier pyramid: deterministic rules (base, widest), small classifiers (middle), model-based judges (narrow top), with "fail closed" running down the side. Beside it, "Step 0: decide autonomy first (L3)" as a gate in front of the pyramid. Inset: the worked example's inline numeric-grounding guard. Source: C2 §C2.9 and §C2.12.</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>- NeMo Guardrails version; any new Meta guardrail releases - Preview or GA status of Azure Task Adherence</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P10" s="4" t="inlineStr"/>
       <c r="Q10" s="4" t="inlineStr"/>
-      <c r="R10" s="4" t="inlineStr">
+      <c r="R10" s="4" t="inlineStr"/>
+      <c r="S10" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 6 · visual 08_Graphic/linkedin/P06.png</t>
         </is>
@@ -1138,50 +1179,55 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
+          <t>Tools: Four tools behind the tool gateway: read-only attribution results with a snapshot hash, read-only fund reference data, a sandboxed calculator for derived figures, and retrieval of approved commentary.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
           <t>Post 8 (C4, Week 4). **Bridge:** The stack post puts a gateway in front of every tool; the control post decides who is allowed through it, and on whose behalf.</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Open tool protocols made connecting tools easy, and that is exactly why tool governance now matters.</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>Open tool protocols have made it easy to connect an agent to almost anything. That is exactly why tool governance now matters.</t>
         </is>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="K11" s="4" t="n">
         <v>242</v>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>#AgenticAI #APISecurity</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>Layer diagram: agent workflow (L3) → tool-governance sub-layer (gateway, private registry, hash-pinned definitions, policy decision, audit) → tools. Tools are colour-coded read-only (green) versus write (amber, "separate approval"). Callout: "45 servers · 20 models · 36.5% average attack success" with the source. Source: L4 §4.2, §4.9 step 0, §4.13 H3 view.</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>- Whether a newer MCP specification makes authorisation mandatory - AAIF governance status of MCP and A2A - MCPTox figures (cite the paper directly if challenged)</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="O11" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
+      <c r="P11" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P11" s="4" t="inlineStr"/>
       <c r="Q11" s="4" t="inlineStr"/>
-      <c r="R11" s="4" t="inlineStr">
+      <c r="R11" s="4" t="inlineStr"/>
+      <c r="S11" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 7 · visual 08_Graphic/linkedin/P07.png</t>
         </is>
@@ -1215,50 +1261,55 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
+          <t>Identity: A registered agent identity with a named sponsor; it acts on behalf of the analyst with a read-only, minutes-long token; a different portfolio manager approves with step-up authentication.</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
           <t>Post 7 (L4, Week 4). **Bridge:** Once every tool sits behind a gateway, the question is who the agent is, and whose authority it carries.</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>"Who did this?" needs an answer when the actor is an agent.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>"Who did this?" is the first question in every incident review. When the actor is an agent, many logs can answer only with the name of a shared service account.</t>
         </is>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>255</v>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>#IAM #AgenticAI</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>"One attribution chain" graphic: analyst signs in → token exchange (on behalf of analyst, read-only scope, minutes TTL) → agent identity (sponsor named) → gateway policy decision → tool → audit event (user · agent · tool · args hash · decision · trace ID) → evidence pack. A separate lane shows the approver (different person, step-up authentication). Source: C4 §C4.12.</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>- Product names and GA status for Entra Agent ID and Okta Agent SSO - Whether any UK or EU rule now names accountability for AI agents</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="P12" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P12" s="4" t="inlineStr"/>
       <c r="Q12" s="4" t="inlineStr"/>
-      <c r="R12" s="4" t="inlineStr">
+      <c r="R12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 8 · visual 08_Graphic/linkedin/P08.png</t>
         </is>
@@ -1292,50 +1343,55 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
+          <t>Memory: Deliberately little: a versioned glossary and style rules per fund, changed only by an approved pull request, recalled by version hash.</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
           <t>Post 10 (Regulated reality, Week 5). **Bridge:** Memory is where governance gets personal (erasure, retention, reproducibility); the control post steps back to the regulations that frame all of it.</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>What an agent remembers is a governance question before it is a technical one, which is why memory comes last.</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>Memory is the layer I would build last, on purpose. What an agent remembers is a governance question before it is a technical one, and it is the layer I would build last.</t>
         </is>
       </c>
-      <c r="J13" s="4" t="n">
+      <c r="K13" s="4" t="n">
         <v>267</v>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>#AgentMemory #DataProtection</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>The build-order roadmap (plan §12.6) as a horizontal timeline: governance → evaluation and observability → model access (gateway first) → retrieval → workflows → tools → **memory** (highlighted) → optimisation. Inset: a memory write path with a policy gate (DLP screen, allow-list, approval), a subject index and a "forget-by-subject" arrow reaching store, vectors, revisions and backups. Source: L5 §5.9 and §5.12.</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>- ICO guidance (under review following the Data (Use and Access) Act) - Memory product defaults (TTL and pruning) and LangMem release status</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr">
+      <c r="P13" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P13" s="4" t="inlineStr"/>
       <c r="Q13" s="4" t="inlineStr"/>
-      <c r="R13" s="4" t="inlineStr">
+      <c r="R13" s="4" t="inlineStr"/>
+      <c r="S13" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 9 · visual 08_Graphic/linkedin/P09.png</t>
         </is>
@@ -1369,50 +1425,55 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
+          <t>Regulation: The regulatory mapping: not an Annex III use; transparency and literacy duties; model vendors as material outsourcing with exit plans; the agent recorded in the model inventory.</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
           <t>Post 9 (L5, Week 5). **Bridge:** Halfway through the layers, the regulatory frame explains why multi-vendor design and retained evidence stop being optional.</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Concentration risk turns multi-vendor from a preference into a requirement.</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Concentration risk is turning multi-vendor AI from a preference into something close to a requirement.</t>
         </is>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="K14" s="4" t="n">
         <v>267</v>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>#EUAIAct #DORA</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>A timeline from April 2026 to December 2027: 17 Apr 2026 SR 26-2 (GenAI out of scope); 13 Jul 2026 UK CTP designations in force; 2 Aug 2026 GPAI enforcement and Article 50 transparency; 18 Mar 2027 UK material third-party notifications; 2 Dec 2027 EU AI Act Annex III. Beneath it, a two-column panel: "designated for direct oversight: hyperscalers and infrastructure" versus "not designated: model vendors (oversight rests on the firm)". Source: regulatory_facts.json and C8 §C8.11.</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>- Any update to the DORA CTPP list or new UK CTP designations (especially any model vendor) - Whether the US agencies' AI request for information has been published - EU AI Act dates (any further Omnibus changes) and the PS7/26 effective date - "For most asset-management uses, today's live duties are literacy and transparency" is a judgement; keep it phrased as such</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr">
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P14" s="4" t="inlineStr"/>
       <c r="Q14" s="4" t="inlineStr"/>
-      <c r="R14" s="4" t="inlineStr">
+      <c r="R14" s="4" t="inlineStr"/>
+      <c r="S14" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 10 · visual 08_Graphic/linkedin/P10.png</t>
         </is>
@@ -1446,50 +1507,55 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
+          <t>Retrieval store: One store already run by the firm, with three collections (prior commentaries, style guide, approved market notes) and fund-level entitlement filters applied inside the search.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
           <t>Post 12 (C7, Week 6). **Bridge:** The stack post is about retrieving the right passages under real permissions; the control post is about the passages someone else wrote for you.</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>You may not need a vector database, but you do need retrieval you can measure.</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>You may not need a vector database. You do need retrieval you can measure.</t>
         </is>
       </c>
-      <c r="J15" s="4" t="n">
+      <c r="K15" s="4" t="n">
         <v>244</v>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>#VectorSearch #RAG</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>Decision-tree graphic (L6 §6.9): Step 0 non-negotiables (filters inside the search, no unfiltered fallback, rebuild tested) → Step 1 "use what you run" (relational database, search engine, document database, object-store tier) → Step 2 three triggers → Step 3 dedicated engine. A side panel contrasts "filter after ranking + fallback = leakage" with "filter inside search + hard empty result".</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>- pgvector version and any new CVEs - Pinecone Nexus and Weaviate licence status</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="O15" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O15" s="4" t="inlineStr">
+      <c r="P15" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P15" s="4" t="inlineStr"/>
       <c r="Q15" s="4" t="inlineStr"/>
-      <c r="R15" s="4" t="inlineStr">
+      <c r="R15" s="4" t="inlineStr"/>
+      <c r="S15" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 11 · visual 08_Graphic/linkedin/P11.png</t>
         </is>
@@ -1523,50 +1589,55 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
+          <t>AI security: Defence in depth against a poisoned market note: nothing to hijack, numbers that cannot be rewritten, retrieved text marked as data, chunk screening, canary documents and human approval.</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
           <t>Post 11 (L6, Week 6). **Bridge:** Retrieval brings back passages; some were written by someone who wants your agent to act on them.</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Every retrieved document is untrusted input. Indirect prompt injection is a supply-chain problem.</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>A language model follows instructions it finds in any text it reads. Give it tools, and those instructions become actions.</t>
         </is>
       </c>
-      <c r="J16" s="4" t="n">
+      <c r="K16" s="4" t="n">
         <v>264</v>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="L16" s="4" t="inlineStr">
         <is>
           <t>#AISecurity #PromptInjection</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>Venn diagram with three circles: untrusted input, sensitive data, outbound channel. The centre is marked "never in one agent". Around it, a defence-in-depth ring for the worked example: deterministic workflow, numeric check, data marking, chunk screening, canary documents, human approval. Source: C7 §C7.9 step 0 and §C7.12.</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>- Any new findings on the March 2026 package compromise (intrusion vector is reported two ways) - Acquisition statuses in the security list</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O16" s="4" t="inlineStr">
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
-      <c r="R16" s="4" t="inlineStr">
+      <c r="R16" s="4" t="inlineStr"/>
+      <c r="S16" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 12 · visual 08_Graphic/linkedin/P12.png</t>
         </is>
@@ -1600,50 +1671,55 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
+          <t>Retrieval quality: Two-stage retrieval of comparable past commentary (embed and rerank), with both model versions pinned and tagged on every vector.</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
           <t>Post 14 (C5, Week 7). **Bridge:** The stack post ends on "the embedding version is production configuration"; the control post extends that to prompts and every other setting that changes outputs.</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>Retrieval quality is a two-stage problem, and it is easy to tune only one stage.</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>Retrieval quality is a two-stage problem, and it is easy to tune only one stage.</t>
         </is>
       </c>
-      <c r="J17" s="4" t="n">
+      <c r="K17" s="4" t="n">
         <v>246</v>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>#InformationRetrieval #RAG</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>Funnel diagram: "corpus → stage 1 (embed, k = 50–100, measure recall@k) → stage 2 (rerank, measure nDCG@10) → top passages to the model". Below it, a small "version tag" icon on each vector and a two-index migration strip (old index live, new index shadow, regression gate, cut-over). Source: L7 §7.3 and §7.9 step 6.</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>- "Every vendor except OpenAI offers both" (check for a new OpenAI reranker) - Current model versions if any are named in replies</t>
         </is>
       </c>
-      <c r="N17" s="4" t="inlineStr">
+      <c r="O17" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O17" s="4" t="inlineStr">
+      <c r="P17" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P17" s="4" t="inlineStr"/>
       <c r="Q17" s="4" t="inlineStr"/>
-      <c r="R17" s="4" t="inlineStr">
+      <c r="R17" s="4" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 13 · visual 08_Graphic/linkedin/P13.png</t>
         </is>
@@ -1677,50 +1753,55 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
+          <t>Configuration: A release manifest per monthly cycle (prompt set, model pins, retrieval settings, tool list, guard policy, eval thresholds), approved by pull request with a second approver and gated by the eval suite.</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
           <t>Post 13 (L7, Week 7). **Bridge:** If the embedding version is production configuration, so is the prompt, and both need versioning, review and rollback.</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Embedding versions and prompts are both production configuration, so they need versioning, review and rollback.</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>A one-sentence edit to a prompt can change outputs as much as a model upgrade. Few organisations would let a model upgrade ship without review. Many let prompts change in a web console.</t>
         </is>
       </c>
-      <c r="J18" s="4" t="n">
+      <c r="K18" s="4" t="n">
         <v>252</v>
       </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>#LLMOps #ChangeManagement</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
+      <c r="M18" s="4" t="inlineStr">
         <is>
           <t>A "release manifest" card for the worked example (illustrative values): prompt set version, drafting model pinned to a dated version, fallback model, embedding and reranker versions, top-k, read-only tool list, guardrail policy version, eval threshold set. Arrows show pull request → second approver → eval gate → tagged release → registry label → trace stamped with version. Source: C5 §C5.12.</t>
         </is>
       </c>
-      <c r="M18" s="4" t="inlineStr">
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>- LaunchDarkly product name (AgentControl) - Langfuse and Promptfoo ownership status</t>
         </is>
       </c>
-      <c r="N18" s="4" t="inlineStr">
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O18" s="4" t="inlineStr">
+      <c r="P18" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="inlineStr">
+      <c r="R18" s="4" t="inlineStr"/>
+      <c r="S18" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 14 · visual 08_Graphic/linkedin/P14.png</t>
         </is>
@@ -1754,50 +1835,55 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
+          <t>Ingestion: Three corpora ingested under a control envelope: dual-parsed factsheet tables reconciled to the engine, prior commentaries with their permissions, and market notes from the approved register only.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
           <t>Post 16 (C3, Week 8). **Bridge:** The stack post shows that quality is decided at ingestion; the control post shows that residency and privacy are decided there too.</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Some of the most convincing "hallucinations" in enterprise retrieval start in a PDF table parser, not in the model.</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>Some of the most convincing "hallucinations" in enterprise retrieval systems are not the model's fault. They start in a table parser.</t>
         </is>
       </c>
-      <c r="J19" s="4" t="n">
+      <c r="K19" s="4" t="n">
         <v>236</v>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="L19" s="4" t="inlineStr">
         <is>
           <t>#RAG #DataQuality</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>Pipeline diagram: source register → acquisition → classification/DLP → parser (drawn as a swappable cartridge) → "metadata envelope" stamped on each chunk (source, version, ACL, classification, parser manifest, lineage ID) → index gate ("no envelope, no index"). A red side-path shows "parsed numbers = context only"; a green path shows "authoritative figures via read-only tool". Source: L8 §8.9 and the six-component control plane in §8.13.</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr">
+      <c r="N19" s="4" t="inlineStr">
         <is>
           <t>- "Ten products assessed; only one carries ACL metadata; none emits lineage" (check for new lineage features) - Mistral OCR and Docling version status if mentioned in replies</t>
         </is>
       </c>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="O19" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O19" s="4" t="inlineStr">
+      <c r="P19" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P19" s="4" t="inlineStr"/>
       <c r="Q19" s="4" t="inlineStr"/>
-      <c r="R19" s="4" t="inlineStr">
+      <c r="R19" s="4" t="inlineStr"/>
+      <c r="S19" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 15 · visual 08_Graphic/linkedin/P15.png</t>
         </is>
@@ -1831,50 +1917,55 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
+          <t>Privacy: One privacy service called at six points: client names and mandates tokenised before any model call, detected again in output, re-identified only for the reviewing manager.</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
           <t>Post 15 (L8, Week 8). **Bridge:** If quality is decided at ingestion, so are residency and privacy; a filter at the prompt arrives too late.</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>Data residency and PII decisions are made at ingestion, not at the prompt.</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>One analyst question can place the same client identifier in seven places: a prompt, a retrieved chunk, a tool result, a provider's processing region, a trace store, an evaluation dataset and a memory record.</t>
         </is>
       </c>
-      <c r="J20" s="4" t="n">
+      <c r="K20" s="4" t="n">
         <v>252</v>
       </c>
-      <c r="K20" s="4" t="inlineStr">
+      <c r="L20" s="4" t="inlineStr">
         <is>
           <t>#DataProtection #PrivacyEngineering</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="M20" s="4" t="inlineStr">
         <is>
           <t>"Seven copies" diagram: one client identifier at the centre with arrows to seven stores (prompt, chunk, tool result, provider region, trace store, eval set, memory). Overlay six numbered enforcement points (E1 ingestion to E6 trace export) all calling one "privacy service" box. Inset: a draft showing CLIENT_A / MANDATE_1 placeholders instead of names. Source: C3 §C3.2, §C3.9 step 0, §C3.12.</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr">
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>- Status of the DPF appeal C-703/25 P - Presidio governance and licence - Purview DSPM licensing statement</t>
         </is>
       </c>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O20" s="4" t="inlineStr">
+      <c r="P20" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="4" t="inlineStr"/>
-      <c r="R20" s="4" t="inlineStr">
+      <c r="R20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 16 · visual 08_Graphic/linkedin/P16.png</t>
         </is>
@@ -1908,50 +1999,55 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
+          <t>Evaluation: The evaluation plane: numeric faithfulness (blocking), groundedness, style, trajectory, and a regression suite of 24 to 36 months of approved commentaries, all on one firm-owned telemetry spine.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
           <t>Post 18 (C8, Week 9). **Bridge:** The stack post argues that evaluation must exist from day one; the control post shows that the same eval suite, run independently and kept, is the validation evidence a model-risk function needs.</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>The layer that ages slowest is the one most teams build last, and evals added after go-live measure the damage, not the quality.</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>Most diagrams of the AI stack put evaluation in the last box. It is the layer that ages slowest — and the one most teams build last.</t>
         </is>
       </c>
-      <c r="J21" s="4" t="n">
+      <c r="K21" s="4" t="n">
         <v>261</v>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>#AIEvaluation #LLMOps</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr">
+      <c r="M21" s="4" t="inlineStr">
         <is>
           <t>Two-panel diagram. Left: the popular nine-layer stack diagram with "Evals and observability" as the last box. Right: the same stack with evaluation and observability redrawn as a vertical plane running alongside every layer, labelled "firm-owned telemetry and evidence spine", with products drawn as replaceable plug-ins. A small callout shows the one metric: "Numeric faithfulness: 100%, any miss blocks." Source: L9 §9.13 and the H8 provisional view.</t>
         </is>
       </c>
-      <c r="M21" s="4" t="inlineStr">
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>- Arize/Dynatrace completion and the Langfuse/ClickHouse status - Whether OpenAI's Promptfoo acquisition has closed - OpenTelemetry GenAI conventions still at "Development" - The "five of the eleven" count, against the final L9 table</t>
         </is>
       </c>
-      <c r="N21" s="4" t="inlineStr">
+      <c r="O21" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O21" s="4" t="inlineStr">
+      <c r="P21" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P21" s="4" t="inlineStr"/>
       <c r="Q21" s="4" t="inlineStr"/>
-      <c r="R21" s="4" t="inlineStr">
+      <c r="R21" s="4" t="inlineStr"/>
+      <c r="S21" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 17 · visual 08_Graphic/linkedin/P17.png</t>
         </is>
@@ -1985,50 +2081,55 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
+          <t>Governance: The inventory entry for the use case and an evidence pack per approved commentary, keyed by one trace ID, written to an immutable archive.</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
           <t>Post 17 (L9, Week 9). **Bridge:** The stack post's eval suite becomes the control post's validation evidence, but only if someone independent challenges it, it is versioned, and it is retained.</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>Your eval suite *is* your validation evidence. What model-risk discipline means when the "model" is an agent and the main US guidance has stepped aside.</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
         <is>
           <t>In April, the US supervisory guidance that had shaped model risk management since 2011 was replaced. Its successor, SR 26-2, places generative and agentic AI expressly outside its scope.</t>
         </is>
       </c>
-      <c r="J22" s="4" t="n">
+      <c r="K22" s="4" t="n">
         <v>257</v>
       </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>#ModelRisk #AIGovernance</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>One-page "evidence pack" graphic for the worked example: eight tiles (prompt version, model version, data snapshot, tool calls, eval results, approver identity, timestamps, final output), all keyed to one trace ID and feeding an immutable archive. A side panel shows "governed unit = use case" with the model as a vendor component. Source: C8 §C8.12.</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="N22" s="4" t="inlineStr">
         <is>
           <t>- SR 26-2 status, and whether the agencies' AI/GenAI request for information has been published (update the post if it has) - SS1/23 scope statements - Collibra–trail ML completion</t>
         </is>
       </c>
-      <c r="N22" s="4" t="inlineStr">
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O22" s="4" t="inlineStr">
+      <c r="P22" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P22" s="4" t="inlineStr"/>
       <c r="Q22" s="4" t="inlineStr"/>
-      <c r="R22" s="4" t="inlineStr">
+      <c r="R22" s="4" t="inlineStr"/>
+      <c r="S22" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 18 · visual 08_Graphic/linkedin/P18.png</t>
         </is>
@@ -2062,50 +2163,55 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
+          <t>Assembled: All eighteen pieces assembled into one request trace, with a 'may / must never' list in which every 'never' names the component that enforces it.</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
           <t>Post 20 (Start small, Week 10). **Bridge:** The stack post shows the full worked example and its "never" list; the control post shows the minimum platform needed to run it, and what to leave out.</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>What the attribution-commentary agent must never do matters more than what it can do.</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>For nine weeks one example has run underneath this series: an agent that drafts the monthly performance-attribution commentary for a multi-asset fund, with a portfolio manager approving every draft. It is generic and illustrative. Here it is in one place.</t>
         </is>
       </c>
-      <c r="J23" s="4" t="n">
+      <c r="K23" s="4" t="n">
         <v>265</v>
       </c>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>#AgenticAI #AIGovernance</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
+      <c r="M23" s="4" t="inlineStr">
         <is>
           <t>Two-column "may / must never" table for the worked example. Each "never" row has its enforcing component in a coloured chip (read-only tool, numeric comparator, approval interrupt, allow-list, tokenisation, entitlement filter, version pin). Beneath it, the eight-tile evidence pack keyed to one trace ID. Source: synthesis VI.3 and VI.4. Label: "generic, illustrative".</t>
         </is>
       </c>
-      <c r="M23" s="4" t="inlineStr">
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>- No product or regulatory facts in the body. Check that the first comment's per-cloud examples match the final document.</t>
         </is>
       </c>
-      <c r="N23" s="4" t="inlineStr">
+      <c r="O23" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O23" s="4" t="inlineStr">
+      <c r="P23" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P23" s="4" t="inlineStr"/>
       <c r="Q23" s="4" t="inlineStr"/>
-      <c r="R23" s="4" t="inlineStr">
+      <c r="R23" s="4" t="inlineStr"/>
+      <c r="S23" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 19 · visual 08_Graphic/linkedin/P19.png</t>
         </is>
@@ -2139,50 +2245,55 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
+          <t>Minimum go-live: The build order for real: governance and evaluation first, then the gateway, retrieval, the workflow and one read-only tool; memory and everything on the 'not yet' list waits for evidence.</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
           <t>Post 19 (Worked example, Week 10). **Bridge:** The stack post's agent needs a platform; the control post argues that the minimum platform, plus a published "not yet" list, is the right first release.</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>The most valuable part of a reference architecture is the "do not build yet" list.</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="J24" s="4" t="inlineStr">
         <is>
           <t>The most valuable page in a reference architecture is often the "do not build yet" list.</t>
         </is>
       </c>
-      <c r="J24" s="4" t="n">
+      <c r="K24" s="4" t="n">
         <v>264</v>
       </c>
-      <c r="K24" s="4" t="inlineStr">
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t>#EnterpriseArchitecture #AgenticAI</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>Two panels. Left, "Build now": the Stack D minimum as a compact stack (gateway ×2, identity, manifest, checks, eval suite, one store, one workflow, two models). Right, "Do NOT build yet": the not-yet items as greyed-out tiles, each with a one-word trigger for revisiting it ("evidence", "load test", "use case"). Source: synthesis Part VII, Stack D.</t>
         </is>
       </c>
-      <c r="M24" s="4" t="inlineStr">
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>- The not-yet list against the final Part VII and the Part XI tiers (anything promoted from Experimental)</t>
         </is>
       </c>
-      <c r="N24" s="4" t="inlineStr">
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O24" s="4" t="inlineStr">
+      <c r="P24" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P24" s="4" t="inlineStr"/>
       <c r="Q24" s="4" t="inlineStr"/>
-      <c r="R24" s="4" t="inlineStr">
+      <c r="R24" s="4" t="inlineStr"/>
+      <c r="S24" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 20 · visual 08_Graphic/linkedin/P20.png</t>
         </is>
@@ -2216,50 +2327,55 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
+          <t>Build or buy: A build, hybrid or buy decision for each of the seventeen components: build the evidence store, configuration and tools; buy models, serving and security tooling; hybrid elsewhere.</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
           <t>Post 22 (Where not to abstract, Week 11). **Bridge:** The stack post says to own a thin interface in front of what you buy; the control post warns against owning too many interfaces.</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>Build where you differentiate, buy where you would only be maintaining.</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="J25" s="4" t="inlineStr">
         <is>
           <t>Build where you differentiate. Buy where you would only be maintaining.</t>
         </is>
       </c>
-      <c r="J25" s="4" t="n">
+      <c r="K25" s="4" t="n">
         <v>257</v>
       </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="L25" s="4" t="inlineStr">
         <is>
           <t>#EnterpriseArchitecture #BuildVsBuy</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="M25" s="4" t="inlineStr">
         <is>
           <t>Three-column board, "Build · Hybrid · Buy", with the 17 layers and controls placed as cards (for example, Build: tool servers, configuration of record, evidence store; Hybrid: gateway, guardrails, privacy, evaluation, retrieval optimisation; Buy: security tooling, foundation models, serving access). A separate red card reads "Do not build yet: fine-tuning". Source: synthesis Part VIII table.</t>
         </is>
       </c>
-      <c r="M25" s="4" t="inlineStr">
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>- No dated facts in the body. Check the Article 25 wording if challenged ("can, in some cases").</t>
         </is>
       </c>
-      <c r="N25" s="4" t="inlineStr">
+      <c r="O25" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O25" s="4" t="inlineStr">
+      <c r="P25" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P25" s="4" t="inlineStr"/>
       <c r="Q25" s="4" t="inlineStr"/>
-      <c r="R25" s="4" t="inlineStr">
+      <c r="R25" s="4" t="inlineStr"/>
+      <c r="S25" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 21 · visual 08_Graphic/linkedin/P21.png</t>
         </is>
@@ -2293,50 +2409,55 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
+          <t>Thin interfaces: Thin firm-owned interfaces where switching is likely (routing contract, telemetry, datasets, privacy, retrieval) and none around the agent framework.</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
           <t>Post 21 (Build vs buy, Week 11). **Bridge:** The stack post's thin firm-owned interfaces are the right default; the control post names where adding one is the mistake.</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>Frameworks on top of frameworks.</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="J26" s="4" t="inlineStr">
         <is>
           <t>Abstraction is how an architecture stays reversible. Too much of it is how an architecture stops moving.</t>
         </is>
       </c>
-      <c r="J26" s="4" t="n">
+      <c r="K26" s="4" t="n">
         <v>254</v>
       </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="L26" s="4" t="inlineStr">
         <is>
           <t>#SoftwareArchitecture #AgenticAI</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="M26" s="4" t="inlineStr">
         <is>
           <t>Two lists side by side. "Abstract (thin, firm-owned)": routing contract, telemetry collector, datasets, credentials, policy, retrieval interface, embed/rerank, privacy API, memory API, config fetch. "Do not over-abstract": agent frameworks, single-workflow plug-ins, plain database access, store-bundled features, vendor model extras. A small strip beneath shows "multi-vendor necessary" versus "multi-vendor only adds complexity". Source: synthesis IX.1–IX.3.</t>
         </is>
       </c>
-      <c r="M26" s="4" t="inlineStr">
+      <c r="N26" s="4" t="inlineStr">
         <is>
           <t>- No dated facts in the body.</t>
         </is>
       </c>
-      <c r="N26" s="4" t="inlineStr">
+      <c r="O26" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O26" s="4" t="inlineStr">
+      <c r="P26" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P26" s="4" t="inlineStr"/>
       <c r="Q26" s="4" t="inlineStr"/>
-      <c r="R26" s="4" t="inlineStr">
+      <c r="R26" s="4" t="inlineStr"/>
+      <c r="S26" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 22 · visual 08_Graphic/linkedin/P22.png</t>
         </is>
@@ -2370,50 +2491,55 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
+          <t>Exit tested: Lock-in accepted knowingly per component, with the firm's own records (evidence, configuration, datasets, credentials) kept out of any vendor's hands, and an index rebuild drilled.</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
           <t>Post 24 (Close, Week 12). **Bridge:** The stack post classifies which dependencies are worth accepting; the control post applies that to the final stack: what I would select, and what I would deliberately leave out.</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>Some lock-in is a good trade, and the skill is knowing which.</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="J27" s="4" t="inlineStr">
         <is>
           <t>Some lock-in is a good trade. The skill is knowing which.</t>
         </is>
       </c>
-      <c r="J27" s="4" t="n">
+      <c r="K27" s="4" t="n">
         <v>257</v>
       </c>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="L27" s="4" t="inlineStr">
         <is>
           <t>#VendorRisk #EnterpriseArchitecture</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr">
+      <c r="M27" s="4" t="inlineStr">
         <is>
           <t>Heat-map table: the 17 layers and controls as rows; columns "acceptable", "manageable", "unacceptable"; each cell a short phrase from the synthesis table (vendor names removed). A highlighted band across the "unacceptable" column reads "the firm's own records: evidence, configuration, datasets, credentials". Source: synthesis IX.4.</t>
         </is>
       </c>
-      <c r="M27" s="4" t="inlineStr">
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>- Lock-in categories against the final Part IX.4 table - Any new ownership change in a "manageable" category</t>
         </is>
       </c>
-      <c r="N27" s="4" t="inlineStr">
+      <c r="O27" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O27" s="4" t="inlineStr">
+      <c r="P27" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P27" s="4" t="inlineStr"/>
       <c r="Q27" s="4" t="inlineStr"/>
-      <c r="R27" s="4" t="inlineStr">
+      <c r="R27" s="4" t="inlineStr"/>
+      <c r="S27" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 23 · visual 08_Graphic/linkedin/P23.png</t>
         </is>
@@ -2447,50 +2573,55 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
+          <t>Signed off: The final selection: a firm-owned control and evidence plane, with replaceable components beneath it, and a published list of what was deliberately not selected.</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
           <t>Post 23 (Which lock-in is acceptable, Week 12). **Bridge:** The stack post's lock-in classification is the filter; the control post shows what passes through it, what does not, and what leading the change actually requires.</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>The full stack on one page, plus a lesson about leading the transformation.</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>Twelve weeks ago this series started from a popular diagram of the AI stack. On this review, 39 of its 80 product tiles were out of date. The diagram was a catalogue. The enterprise problem is a control system.</t>
         </is>
       </c>
-      <c r="J28" s="4" t="n">
+      <c r="K28" s="4" t="n">
         <v>269</v>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="L28" s="4" t="inlineStr">
         <is>
           <t>#EnterpriseArchitecture #AIGovernance</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t>The one-page architecture from synthesis I.2, with vendor names removed: control plane (C1–C8 with the L9 evidence plane) across the top; agent, knowledge and model planes beneath. To the right, a short "Deliberately not selected" column with the categories from XI.5 and XI.7. Optional carousel: slide 1 the popular stack diagram with 39 tiles flagged; slide 2 the one-page architecture; slide 3 the twelve decisions; slide 4 "not selected".</t>
         </is>
       </c>
-      <c r="M28" s="4" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>- The final Part XI lists (avoid and monitor), especially any item that has changed tier since October 2026 - Ownership and status changes across the products in the first comment</t>
         </is>
       </c>
-      <c r="N28" s="4" t="inlineStr">
+      <c r="O28" s="4" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="O28" s="4" t="inlineStr">
+      <c r="P28" s="4" t="inlineStr">
         <is>
           <t>Not required (CP4b)</t>
         </is>
       </c>
-      <c r="P28" s="4" t="inlineStr"/>
       <c r="Q28" s="4" t="inlineStr"/>
-      <c r="R28" s="4" t="inlineStr">
+      <c r="R28" s="4" t="inlineStr"/>
+      <c r="S28" s="4" t="inlineStr">
         <is>
           <t>07_LinkedIn/LinkedIn_Series.docx, Post 24 · visual 08_Graphic/linkedin/P24.png</t>
         </is>
@@ -2498,7 +2629,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="N4:N28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O4:O28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Draft,Anecdote added,Scheduled,Published,Skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Content calendar and series document rebuilt: 33 posts over 17 weeks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYt6k15P64MhHqeyveeQ6D
</commit_message>
<xml_diff>
--- a/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
+++ b/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S28"/>
+  <dimension ref="A1:S36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2627,9 +2627,633 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Views post</t>
+        </is>
+      </c>
+      <c r="D29" s="5">
+        <f>IF($E$1="","",$E$1+84)</f>
+        <v/>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>One stack, seven lenses: who builds it, runs it or sells into it</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Post 26 (TS, Week 13). **Bridge:** The opener names the seven lenses and what each weights most; the next post takes the first of them, the company that runs GenAI inside a service its customers pay for.</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>Same stack, different owner of the control plane, and that is what changes the advice.</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>If you build GenAI into what you sell, run it for customers, or sell into someone else's stack, the next eight posts are for you.</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="n">
+        <v>269</v>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>#GenerativeAI #EnterpriseArchitecture</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>The seven views on one card: one row each for FS, TS, SW, SU, AT, DV and AG, in that order, with who it is for in a few words, the eight criterion weights as a compact grid (the heaviest per row in gold), the role the reader plays (deployer, operator, manufacturer, supplier) and core candidates of 138. Source: `views.json` and §3 of Parts XIII–XVIII.</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>- Weights and core-candidate counts against the published `05_Data/views.xlsx` (they change if the scores are refreshed) - The PLD date and NIS2 scope wording in the first comment</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="P29" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="Q29" s="4" t="inlineStr"/>
+      <c r="R29" s="4" t="inlineStr"/>
+      <c r="S29" s="4" t="inlineStr">
+        <is>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 25 · visual 08_Graphic/linkedin/P25.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Views post</t>
+        </is>
+      </c>
+      <c r="D30" s="5">
+        <f>IF($E$1="","",$E$1+86)</f>
+        <v/>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Technology service provider: margin, uptime and tenant isolation change the defaults</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr"/>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Post 25 (the opener, Week 13). **Bridge:** The opener said the weights move with the reader; this post shows what moves when every model call is cost of goods sold and every customer shares one estate.</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>Same plane as a bank's, but every element of it tenant-aware, metered and sold.</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>If you run GenAI inside a service your customers pay for, this one is for you.</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>263</v>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>#SaaS #EnterpriseArchitecture</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>Weights compared with the regulated-FS view (eight paired bars, FS against TS, with the change marked), then the three layers whose advice changes most, in layer order: L1 models (the second vendor becomes a live capacity route), L6 stores (tenant isolation replaces entitlement within one firm), C6 FinOps (from reporting to gross-margin control). A strip states what stays (gateway of record, day-one evaluation, approval-gated workflows, configuration in source control) and the core-candidate cou</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>- Batch, cache and Flex pricing at each vendor (volatile) - Anthropic's Usage Policy effective 12 November 2026, for the suspension wording</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="P30" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="Q30" s="4" t="inlineStr"/>
+      <c r="R30" s="4" t="inlineStr"/>
+      <c r="S30" s="4" t="inlineStr">
+        <is>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 26 · visual 08_Graphic/linkedin/P26.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Views post</t>
+        </is>
+      </c>
+      <c r="D31" s="5">
+        <f>IF($E$1="","",$E$1+91)</f>
+        <v/>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Software product company: your stack has to run where your customer runs</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Post 28 (SU, Week 14). **Bridge:** A software company ships into estates it does not control; a start-up builds its own, fast. The next post shows what changes when runway, not the customer's estate, is the constraint.</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>What is fine to run internally can be impossible to ship.</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>If you ship software with GenAI built in that your customers install and run, this one is for you.</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="n">
+        <v>263</v>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>#SoftwareEngineering #EnterpriseArchitecture</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>Weights compared with the regulated-FS view (eight paired bars, FS against SW), then the three layers whose advice changes most: L1 models (a support matrix and a bundled open-weight model replace the two-vendor portfolio), C1 gateway (routed by the customer's gateway, not the gateway of record), C7 security (sign and patch every shipped copy for the support period, with a redistribution gate in CI). A strip states "own a release plane, not a control plane" and the core-candidate count, 45 to 48</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>- Hosted-model retirement dates and the licences of the bundled open-weight models - CRA guidance and delegated acts (not read in full at drafting)</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="P31" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="Q31" s="4" t="inlineStr"/>
+      <c r="R31" s="4" t="inlineStr"/>
+      <c r="S31" s="4" t="inlineStr">
+        <is>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 27 · visual 08_Graphic/linkedin/P27.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Views post</t>
+        </is>
+      </c>
+      <c r="D32" s="5">
+        <f>IF($E$1="","",$E$1+93)</f>
+        <v/>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Start-up: speed and runway first, with exits kept open cheaply</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr"/>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Post 27 (SW, Week 14). **Bridge:** The software company ships into estates it does not control; the start-up controls its own, and has to decide how much of the regulated firm's plane it can afford in its first fortnight.</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>Each control must cost days, not quarters, and still keep the exits open.</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>If you are building an AI-native product with a small team and a runway to watch, this one is for you.</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>272</v>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>#Startups #GenerativeAI</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>Weights compared with the regulated-FS view (eight paired bars, FS against SU), then the three layers whose advice changes most: L1 models (one primary vendor plus a second qualified, first-party access allowed), L6 stores (tenant isolation becomes the first control problem), C4 identity (hosted customer identity, not a workforce directory). A strip lists the first-fortnight four and the core-candidate count, 45 to 57. Source: Part XV.1, XV.3, XV.4 and XV.5.</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>- Credit programme terms and router fees (volatile; quarterly) - The current LiteLLM release line and advisory</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="P32" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="Q32" s="4" t="inlineStr"/>
+      <c r="R32" s="4" t="inlineStr"/>
+      <c r="S32" s="4" t="inlineStr">
+        <is>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 28 · visual 08_Graphic/linkedin/P28.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Views post</t>
+        </is>
+      </c>
+      <c r="D33" s="5">
+        <f>IF($E$1="","",$E$1+98)</f>
+        <v/>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>AI-tools start-up: to be bought, fit the buyer's control plane</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Post 30 (DV, Week 15). **Bridge:** A tools start-up sells one component of the buyer's control plane; an agentic software-delivery start-up sells a workload that runs inside it and inside the buyer's delivery chain at once.</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>You win by designing for the buyer's "everything beneath the plane is replaceable" posture, not against it.</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>If your start-up sells a gateway, guardrail, privacy, evaluation, retrieval or governance tool to enterprises, this one is for you.</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>271</v>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>#Startups #AIGovernance</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>The integration contract, layer by layer then control by control: seventeen rows L1 → L9 then C1 → C8, each with what the buyer's stack expects and the interface the product should offer. Boxes beneath give the single test (evidence pack with the product in the path; removal by one route and one manifest entry) and the three delivery forms from one build. Source: Part XVI.4 and XVI.5.</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>- Closing status of the announced acquisitions (Promptfoo, OpenRouter) and any new ones in the tool categories - OpenTelemetry GenAI conventions release status</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="P33" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="Q33" s="4" t="inlineStr"/>
+      <c r="R33" s="4" t="inlineStr"/>
+      <c r="S33" s="4" t="inlineStr">
+        <is>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 29 · visual 08_Graphic/linkedin/P29.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Views post</t>
+        </is>
+      </c>
+      <c r="D34" s="5">
+        <f>IF($E$1="","",$E$1+100)</f>
+        <v/>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Agentic-SDLC start-up: code confidentiality and audit trails decide the deal</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr"/>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Post 29 (AT, Week 15). **Bridge:** A tools start-up is a call-out inside the buyer's plane; a coding-agent start-up runs inside that plane and the buyer's delivery chain at once, holding the most sensitive asset the buyer has.</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Trust is earned in the pull request, not the demo.</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>If your start-up sells coding agents, AI code review, test generation or migration agents to enterprise engineering teams, this one is for you.</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>265</v>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>#DevOps #AIGovernance</t>
+        </is>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>The integration contract, layer by layer then control by control: seventeen rows L1 → L9 then C1 → C8, with what the buyer's stack expects and what the coding agent must do. A band beneath shows the pull-request boundary (agent branch, the customer's CI and scanning, a named human merges), beside a box of what the agent must never do. Source: Part XVII.4 and XVII.5.</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>- Retention terms per model and tool, including the end-of-2026 Copilot exemption for Claude Fable - Ownership and end-of-sale events among the coding-agent incumbents</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="P34" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="Q34" s="4" t="inlineStr"/>
+      <c r="R34" s="4" t="inlineStr"/>
+      <c r="S34" s="4" t="inlineStr">
+        <is>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 30 · visual 08_Graphic/linkedin/P30.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Views post</t>
+        </is>
+      </c>
+      <c r="D35" s="5">
+        <f>IF($E$1="","",$E$1+105)</f>
+        <v/>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Agent-provider start-up: an agent the customer can't govern isn't bought</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Post 32 (Close, Week 16). **Bridge:** The agent start-up is the hardest case of fitting someone else's control plane; the close asks what survives across all seven lenses once the owner of the plane changes.</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Capability wins the demo; governance fit wins the purchase.</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>If your start-up sells agents that do work inside a customer's business, this one is for you.</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>264</v>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>#AIAgents #AIGovernance</t>
+        </is>
+      </c>
+      <c r="M35" s="4" t="inlineStr">
+        <is>
+          <t>The integration contract, layer by layer then control by control: seventeen rows L1 → L9 then C1 → C8, with what the customer's stack expects and the interface the agent must offer, the seven clauses marked against the rows they cover. A box gives the three-part test (audit every output, revoke with one identity, switch model with one route). Source: Part XVIII.4 and XVIII.5.</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>- ID-JAG draft status (draft -04 expires 22 November 2026) and MCP authorisation changes - OpenTelemetry GenAI conventions release status; marketplace listing rules</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="P35" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="Q35" s="4" t="inlineStr"/>
+      <c r="R35" s="4" t="inlineStr"/>
+      <c r="S35" s="4" t="inlineStr">
+        <is>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 31 · visual 08_Graphic/linkedin/P31.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Views post</t>
+        </is>
+      </c>
+      <c r="D36" s="5">
+        <f>IF($E$1="","",$E$1+107)</f>
+        <v/>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Close: what doesn't change across all seven lenses</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr"/>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>Post 31 (AG, Week 16). **Bridge:** The agent start-up showed the plane from the guest's side; the close lays all seven lenses over the seventeen layers and controls and keeps what none of them changes.</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>Lenses change the defaults. They do not change the discipline.</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>If you have followed one lens of this run, or all seven, this post closes it.</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>269</v>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>#EnterpriseArchitecture #AIGovernance</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>A heat map: the seventeen layers and controls as rows (L1 → L9 then C1 → C8), the seven views as columns (FS as the baseline, then TS, SW, SU, AT, DV, AG), each cell shaded "holds", "adjusted" or "changes" by the author's reading of each Part's layer-by-layer table. Rows where no lens changes the answer are marked; a side panel lists the six things that hold in all seven. Source: §5 of Parts XIII–XVIII against synthesis I.2.</t>
+        </is>
+      </c>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>- Whether the PLD date has passed when the post goes out (adjust "From 9 December 2026" to "Since 9 December 2026") - Any change to the view Parts' layer tables since drafting, which would change the shading</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="P36" s="4" t="inlineStr">
+        <is>
+          <t>Not required (CP4b)</t>
+        </is>
+      </c>
+      <c r="Q36" s="4" t="inlineStr"/>
+      <c r="R36" s="4" t="inlineStr"/>
+      <c r="S36" s="4" t="inlineStr">
+        <is>
+          <t>07_LinkedIn/LinkedIn_Series.docx, Post 32 · visual 08_Graphic/linkedin/P32.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="O4:O28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O4:O36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Draft,Anecdote added,Scheduled,Published,Skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Full rebuild: dataset, views, figures, explorer, LinkedIn calendar and series, deck (38 slides) and deck PDF, master, print and Kindle edition (Interior.docx), LinkedIn book with Part IV, appendix; no ZIP, no PDF from any Word document
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYt6k15P64MhHqeyveeQ6D
</commit_message>
<xml_diff>
--- a/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
+++ b/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>The logos move faster than any diagram; the controls around them are what last.</t>
+          <t>The logos move every quarter; the controls around them are what last.</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>- The counts (140 products, 1,255 sources, 39 of 80 tiles) against the final published edition - The planned date of Post 1 (set in the content calendar)</t>
+          <t>- The counts (140 products, 138 scored, 1,449 sources) against the final published edition - The planned date of Post 1 (set in the content calendar)</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
@@ -2014,11 +2014,11 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Most diagrams of the AI stack put evaluation in the last box. It is the layer that ages slowest — and the one most teams build last.</t>
+          <t>Evaluation usually sits in the last box of the AI stack. It is the layer that ages slowest — and the one most teams build last.</t>
         </is>
       </c>
       <c r="K21" s="4" t="n">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>Two-panel diagram. Left: the popular nine-layer stack diagram with "Evals and observability" as the last box. Right: the same stack with evaluation and observability redrawn as a vertical plane running alongside every layer, labelled "firm-owned telemetry and evidence spine", with products drawn as replaceable plug-ins. A small callout shows the one metric: "Numeric faithfulness: 100%, any miss blocks." Source: L9 §9.13 and the H8 provisional view.</t>
+          <t>Two-panel diagram. Left: a generic pipeline view of the nine layers with "Evals and observability" as the last box, usually built last. Right: the new baseline, with evaluation and observability redrawn as a vertical plane running alongside every layer, labelled "firm-owned telemetry and evidence spine", with products drawn as replaceable plug-ins. A small callout shows the one metric: "Numeric faithfulness: 100%, any miss blocks." Source: L9 §9.13 and the H8 provisional view.</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr">
@@ -2588,11 +2588,11 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Twelve weeks ago this series started from a popular diagram of the AI stack. On this review, 39 of its 80 product tiles were out of date. The diagram was a catalogue. The enterprise problem is a control system.</t>
+          <t>Twelve weeks ago this series set out to build a new baseline for the enterprise GenAI stack, from the evidence up. The finding held all the way through: this is not a catalogue problem. The enterprise problem is a control system.</t>
         </is>
       </c>
       <c r="K28" s="4" t="n">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>The one-page architecture from synthesis I.2, with vendor names removed: control plane (C1–C8 with the L9 evidence plane) across the top; agent, knowledge and model planes beneath. To the right, a short "Deliberately not selected" column with the categories from XI.5 and XI.7. Optional carousel: slide 1 the popular stack diagram with 39 tiles flagged; slide 2 the one-page architecture; slide 3 the twelve decisions; slide 4 "not selected".</t>
+          <t>The one-page architecture from synthesis I.2, with vendor names removed: control plane (C1–C8 with the L9 evidence plane) across the top; agent, knowledge and model planes beneath. To the right, a short "Deliberately not selected" column with the categories from XI.5 and XI.7. Optional carousel: slide 1 the new baseline at a glance (nine layers, eight controls, 140 products assessed); slide 2 the one-page architecture; slide 3 the twelve decisions; slide 4 "not selected".</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Edition setting: edition.json read by every tool; new_edition.py, check_edition.py; deck counts from dataset_stats.json
</commit_message>
<xml_diff>
--- a/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
+++ b/Enterprise_GenAI_Stack_Oct2026/07_LinkedIn/Content_Calendar.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>The logos move faster than any diagram; the controls around them are what last.</t>
+          <t>The logos move every quarter; the controls around them are what last.</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>- The counts (140 products, 1,255 sources, 39 of 80 tiles) against the final published edition - The planned date of Post 1 (set in the content calendar)</t>
+          <t>- The counts (140 products, 138 scored, 1,449 sources) against the final published edition - The planned date of Post 1 (set in the content calendar)</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
@@ -2014,11 +2014,11 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Most diagrams of the AI stack put evaluation in the last box. It is the layer that ages slowest — and the one most teams build last.</t>
+          <t>Evaluation usually sits in the last box of the AI stack. It is the layer that ages slowest — and the one most teams build last.</t>
         </is>
       </c>
       <c r="K21" s="4" t="n">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>Two-panel diagram. Left: the popular nine-layer stack diagram with "Evals and observability" as the last box. Right: the same stack with evaluation and observability redrawn as a vertical plane running alongside every layer, labelled "firm-owned telemetry and evidence spine", with products drawn as replaceable plug-ins. A small callout shows the one metric: "Numeric faithfulness: 100%, any miss blocks." Source: L9 §9.13 and the H8 provisional view.</t>
+          <t>Two-panel diagram. Left: a generic pipeline view of the nine layers with "Evals and observability" as the last box, usually built last. Right: the new baseline, with evaluation and observability redrawn as a vertical plane running alongside every layer, labelled "firm-owned telemetry and evidence spine", with products drawn as replaceable plug-ins. A small callout shows the one metric: "Numeric faithfulness: 100%, any miss blocks." Source: L9 §9.13 and the H8 provisional view.</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr">
@@ -2588,11 +2588,11 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Twelve weeks ago this series started from a popular diagram of the AI stack. On this review, 39 of its 80 product tiles were out of date. The diagram was a catalogue. The enterprise problem is a control system.</t>
+          <t>Twelve weeks ago this series set out to build a new baseline for the enterprise GenAI stack, from the evidence up. The finding held all the way through: this is not a catalogue problem. The enterprise problem is a control system.</t>
         </is>
       </c>
       <c r="K28" s="4" t="n">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>The one-page architecture from synthesis I.2, with vendor names removed: control plane (C1–C8 with the L9 evidence plane) across the top; agent, knowledge and model planes beneath. To the right, a short "Deliberately not selected" column with the categories from XI.5 and XI.7. Optional carousel: slide 1 the popular stack diagram with 39 tiles flagged; slide 2 the one-page architecture; slide 3 the twelve decisions; slide 4 "not selected".</t>
+          <t>The one-page architecture from synthesis I.2, with vendor names removed: control plane (C1–C8 with the L9 evidence plane) across the top; agent, knowledge and model planes beneath. To the right, a short "Deliberately not selected" column with the categories from XI.5 and XI.7. Optional carousel: slide 1 the new baseline at a glance (nine layers, eight controls, 140 products assessed); slide 2 the one-page architecture; slide 3 the twelve decisions; slide 4 "not selected".</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr">

</xml_diff>